<commit_message>
"Update coleta_flow.db and add import service"
</commit_message>
<xml_diff>
--- a/uploads/coletas.xlsx.xlsx
+++ b/uploads/coletas.xlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALIX\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{622B82EB-FA0C-47F3-AAE7-7EC1093E93BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A0A99D-5929-431A-9445-D9B8DC24F144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="125">
   <si>
     <t>7 TON</t>
   </si>
@@ -389,9 +389,6 @@
   </si>
   <si>
     <t xml:space="preserve">Brasil Atacadista - Itinga - Lj </t>
-  </si>
-  <si>
-    <t>CRH</t>
   </si>
   <si>
     <t>92L</t>
@@ -1110,22 +1107,105 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="12" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="13" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1136,91 +1216,22 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="17" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="17" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="12" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1241,23 +1252,6 @@
     <xf numFmtId="14" fontId="3" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="17" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="13" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1265,6 +1259,9 @@
     <xf numFmtId="14" fontId="13" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1778,41 +1775,41 @@
       <c r="M1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="113">
+      <c r="N1" s="120">
         <v>46169</v>
       </c>
-      <c r="O1" s="113"/>
+      <c r="O1" s="120"/>
     </row>
     <row r="2" spans="1:19" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="100" t="s">
+      <c r="A2" s="109" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="101"/>
-      <c r="C2" s="102"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="111"/>
       <c r="D2" s="20" t="s">
         <v>15</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="95" t="s">
+      <c r="F2" s="112" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="96"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="95" t="s">
+      <c r="G2" s="113"/>
+      <c r="H2" s="114"/>
+      <c r="I2" s="112" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="96"/>
-      <c r="K2" s="97"/>
+      <c r="J2" s="113"/>
+      <c r="K2" s="114"/>
       <c r="L2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="109" t="s">
+      <c r="M2" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="N2" s="110"/>
-      <c r="O2" s="111"/>
+      <c r="N2" s="116"/>
+      <c r="O2" s="117"/>
       <c r="P2" s="15" t="s">
         <v>81</v>
       </c>
@@ -1894,7 +1891,7 @@
         <v>seg</v>
       </c>
       <c r="P4" s="19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -2224,10 +2221,10 @@
       <c r="A13" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="B13" s="114" t="s">
+      <c r="B13" s="102" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="114"/>
+      <c r="C13" s="102"/>
       <c r="D13" s="18">
         <v>20</v>
       </c>
@@ -2259,7 +2256,7 @@
         <v>ter</v>
       </c>
       <c r="P13" s="19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="21" x14ac:dyDescent="0.25">
@@ -2267,7 +2264,7 @@
         <v>105</v>
       </c>
       <c r="B14" s="25" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C14" s="26"/>
       <c r="D14" s="30">
@@ -2303,10 +2300,10 @@
     </row>
     <row r="15" spans="1:19" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C15" s="26"/>
       <c r="D15" s="30">
@@ -2345,7 +2342,7 @@
         <v>24</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C16" s="26"/>
       <c r="D16" s="30">
@@ -2384,7 +2381,7 @@
         <v>99</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C17" s="26"/>
       <c r="D17" s="30">
@@ -2461,10 +2458,10 @@
       <c r="A19" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="114" t="s">
+      <c r="B19" s="102" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="115"/>
+      <c r="C19" s="103"/>
       <c r="D19" s="30">
         <v>7</v>
       </c>
@@ -2536,7 +2533,7 @@
         <v>ter</v>
       </c>
       <c r="P20" s="19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:19" s="66" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -2551,32 +2548,32 @@
         <v>15</v>
       </c>
       <c r="E21" s="72"/>
-      <c r="F21" s="116">
+      <c r="F21" s="97">
         <v>46147</v>
       </c>
-      <c r="G21" s="117"/>
+      <c r="G21" s="98"/>
       <c r="H21" s="73"/>
-      <c r="I21" s="116">
+      <c r="I21" s="97">
         <v>46170</v>
       </c>
-      <c r="J21" s="117"/>
+      <c r="J21" s="98"/>
       <c r="K21" s="73"/>
       <c r="L21" s="74">
         <f t="shared" si="3"/>
         <v>23</v>
       </c>
-      <c r="M21" s="118">
+      <c r="M21" s="99">
         <f t="shared" ref="M21:M29" si="28">IF(WEEKDAY((I21+D21))=7,(I21+D21)-1,IF(WEEKDAY((I21+D21))=1,(I21+D21)-2,(I21+D21)))</f>
         <v>46185</v>
       </c>
-      <c r="N21" s="118"/>
+      <c r="N21" s="99"/>
       <c r="O21" s="75" t="str">
         <f t="shared" si="5"/>
         <v>sex</v>
       </c>
       <c r="P21" s="76"/>
-      <c r="Q21" s="120"/>
-      <c r="R21" s="121"/>
+      <c r="Q21" s="107"/>
+      <c r="R21" s="108"/>
     </row>
     <row r="22" spans="1:19" s="66" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="68" t="s">
@@ -2590,344 +2587,344 @@
         <v>15</v>
       </c>
       <c r="E22" s="72"/>
-      <c r="F22" s="116">
+      <c r="F22" s="97">
         <v>46129</v>
       </c>
-      <c r="G22" s="117"/>
+      <c r="G22" s="98"/>
       <c r="H22" s="73"/>
-      <c r="I22" s="116">
+      <c r="I22" s="97">
         <v>46155</v>
       </c>
-      <c r="J22" s="117"/>
+      <c r="J22" s="98"/>
       <c r="K22" s="73"/>
       <c r="L22" s="74">
         <f t="shared" si="3"/>
         <v>26</v>
       </c>
-      <c r="M22" s="118">
+      <c r="M22" s="99">
         <f t="shared" si="28"/>
         <v>46170</v>
       </c>
-      <c r="N22" s="118"/>
+      <c r="N22" s="99"/>
       <c r="O22" s="75" t="str">
         <f t="shared" si="5"/>
         <v>qui</v>
       </c>
       <c r="P22" s="76"/>
-      <c r="Q22" s="120"/>
-      <c r="R22" s="121"/>
+      <c r="Q22" s="107"/>
+      <c r="R22" s="108"/>
     </row>
     <row r="23" spans="1:19" s="87" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="77" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="103" t="s">
+      <c r="B23" s="92" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="104"/>
+      <c r="C23" s="93"/>
       <c r="D23" s="51">
         <v>10</v>
       </c>
       <c r="E23" s="78"/>
-      <c r="F23" s="105">
+      <c r="F23" s="94">
         <v>46164</v>
       </c>
-      <c r="G23" s="106"/>
+      <c r="G23" s="95"/>
       <c r="H23" s="79"/>
-      <c r="I23" s="105">
+      <c r="I23" s="94">
         <v>46171</v>
       </c>
-      <c r="J23" s="106"/>
+      <c r="J23" s="95"/>
       <c r="K23" s="79"/>
       <c r="L23" s="54">
         <f t="shared" ref="L23" si="29">I23-F23</f>
         <v>7</v>
       </c>
-      <c r="M23" s="108">
+      <c r="M23" s="96">
         <f t="shared" si="28"/>
         <v>46181</v>
       </c>
-      <c r="N23" s="108"/>
+      <c r="N23" s="96"/>
       <c r="O23" s="55" t="str">
         <f t="shared" ref="O23" si="30">IFERROR(TEXT(WEEKDAY(M23),"ddd"),"")</f>
         <v>seg</v>
       </c>
       <c r="P23" s="29"/>
-      <c r="Q23" s="120"/>
-      <c r="R23" s="121"/>
+      <c r="Q23" s="107"/>
+      <c r="R23" s="108"/>
       <c r="S23" s="2"/>
     </row>
     <row r="24" spans="1:19" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="77" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="103" t="s">
+      <c r="B24" s="92" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="104"/>
+      <c r="C24" s="93"/>
       <c r="D24" s="51">
         <v>4</v>
       </c>
       <c r="E24" s="78"/>
-      <c r="F24" s="98">
+      <c r="F24" s="122">
         <v>46167</v>
       </c>
-      <c r="G24" s="99"/>
+      <c r="G24" s="123"/>
       <c r="H24" s="80"/>
-      <c r="I24" s="98">
+      <c r="I24" s="122">
         <v>46170</v>
       </c>
-      <c r="J24" s="99"/>
+      <c r="J24" s="123"/>
       <c r="K24" s="79"/>
       <c r="L24" s="54">
         <f>I24-F24</f>
         <v>3</v>
       </c>
-      <c r="M24" s="108">
+      <c r="M24" s="96">
         <f t="shared" si="28"/>
         <v>46174</v>
       </c>
-      <c r="N24" s="108"/>
+      <c r="N24" s="96"/>
       <c r="O24" s="55" t="str">
         <f t="shared" si="5"/>
         <v>seg</v>
       </c>
       <c r="P24" s="81"/>
-      <c r="Q24" s="120"/>
-      <c r="R24" s="121"/>
+      <c r="Q24" s="107"/>
+      <c r="R24" s="108"/>
     </row>
     <row r="25" spans="1:19" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="103" t="s">
+      <c r="B25" s="92" t="s">
         <v>7</v>
       </c>
-      <c r="C25" s="104"/>
+      <c r="C25" s="93"/>
       <c r="D25" s="51">
         <v>5</v>
       </c>
       <c r="E25" s="78"/>
-      <c r="F25" s="105">
+      <c r="F25" s="94">
         <v>46164</v>
       </c>
-      <c r="G25" s="106"/>
+      <c r="G25" s="95"/>
       <c r="H25" s="79"/>
-      <c r="I25" s="105">
+      <c r="I25" s="94">
         <v>46169</v>
       </c>
-      <c r="J25" s="106"/>
+      <c r="J25" s="95"/>
       <c r="K25" s="79"/>
       <c r="L25" s="54">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="M25" s="108">
+      <c r="M25" s="96">
         <f t="shared" si="28"/>
         <v>46174</v>
       </c>
-      <c r="N25" s="108"/>
+      <c r="N25" s="96"/>
       <c r="O25" s="55" t="str">
         <f t="shared" si="5"/>
         <v>seg</v>
       </c>
       <c r="P25" s="29"/>
-      <c r="Q25" s="120"/>
-      <c r="R25" s="121"/>
+      <c r="Q25" s="107"/>
+      <c r="R25" s="108"/>
     </row>
     <row r="26" spans="1:19" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="77" t="s">
-        <v>109</v>
-      </c>
-      <c r="B26" s="103" t="s">
+        <v>108</v>
+      </c>
+      <c r="B26" s="92" t="s">
         <v>41</v>
       </c>
-      <c r="C26" s="104"/>
+      <c r="C26" s="93"/>
       <c r="D26" s="51">
         <v>7</v>
       </c>
       <c r="E26" s="78"/>
-      <c r="F26" s="105">
+      <c r="F26" s="94">
         <v>46161</v>
       </c>
-      <c r="G26" s="106"/>
+      <c r="G26" s="95"/>
       <c r="H26" s="79"/>
-      <c r="I26" s="105">
+      <c r="I26" s="94">
         <v>46168</v>
       </c>
-      <c r="J26" s="106"/>
+      <c r="J26" s="95"/>
       <c r="K26" s="79"/>
       <c r="L26" s="54">
         <f t="shared" ref="L26" si="31">I26-F26</f>
         <v>7</v>
       </c>
-      <c r="M26" s="108">
+      <c r="M26" s="96">
         <f t="shared" ref="M26" si="32">IF(WEEKDAY((I26+D26))=7,(I26+D26)-1,IF(WEEKDAY((I26+D26))=1,(I26+D26)-2,(I26+D26)))</f>
         <v>46175</v>
       </c>
-      <c r="N26" s="108"/>
+      <c r="N26" s="96"/>
       <c r="O26" s="55" t="str">
         <f t="shared" ref="O26" si="33">IFERROR(TEXT(WEEKDAY(M26),"ddd"),"")</f>
         <v>ter</v>
       </c>
       <c r="P26" s="29"/>
-      <c r="Q26" s="120"/>
-      <c r="R26" s="121"/>
+      <c r="Q26" s="107"/>
+      <c r="R26" s="108"/>
     </row>
     <row r="27" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="77" t="s">
         <v>103</v>
       </c>
-      <c r="B27" s="103" t="s">
+      <c r="B27" s="92" t="s">
         <v>104</v>
       </c>
-      <c r="C27" s="104"/>
+      <c r="C27" s="93"/>
       <c r="D27" s="51">
         <v>10</v>
       </c>
       <c r="E27" s="78"/>
-      <c r="F27" s="105">
+      <c r="F27" s="94">
         <v>46161</v>
       </c>
-      <c r="G27" s="106"/>
+      <c r="G27" s="95"/>
       <c r="H27" s="79">
         <v>0</v>
       </c>
-      <c r="I27" s="105">
+      <c r="I27" s="94">
         <v>46170</v>
       </c>
-      <c r="J27" s="106"/>
+      <c r="J27" s="95"/>
       <c r="K27" s="79"/>
       <c r="L27" s="54">
         <f t="shared" si="3"/>
         <v>9</v>
       </c>
-      <c r="M27" s="108">
+      <c r="M27" s="96">
         <f t="shared" ref="M27:M28" si="34">IF(WEEKDAY((I27+D27))=7,(I27+D27)-1,IF(WEEKDAY((I27+D27))=1,(I27+D27)-2,(I27+D27)))</f>
         <v>46178</v>
       </c>
-      <c r="N27" s="108"/>
+      <c r="N27" s="96"/>
       <c r="O27" s="55" t="str">
         <f t="shared" si="5"/>
         <v>sex</v>
       </c>
       <c r="P27" s="29"/>
-      <c r="Q27" s="120"/>
-      <c r="R27" s="121"/>
+      <c r="Q27" s="107"/>
+      <c r="R27" s="108"/>
     </row>
     <row r="28" spans="1:19" s="56" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="48" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B28" s="49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C28" s="50"/>
       <c r="D28" s="51">
         <v>10</v>
       </c>
       <c r="E28" s="52"/>
-      <c r="F28" s="105">
+      <c r="F28" s="94">
         <v>46164</v>
       </c>
-      <c r="G28" s="106"/>
+      <c r="G28" s="95"/>
       <c r="H28" s="53">
         <v>6240</v>
       </c>
-      <c r="I28" s="105">
+      <c r="I28" s="94">
         <v>46171</v>
       </c>
-      <c r="J28" s="106"/>
+      <c r="J28" s="95"/>
       <c r="K28" s="53"/>
       <c r="L28" s="54">
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="M28" s="108">
+      <c r="M28" s="96">
         <f t="shared" si="34"/>
         <v>46181</v>
       </c>
-      <c r="N28" s="108"/>
+      <c r="N28" s="96"/>
       <c r="O28" s="55" t="str">
         <f t="shared" si="5"/>
         <v>seg</v>
       </c>
       <c r="P28" s="29"/>
-      <c r="Q28" s="120"/>
-      <c r="R28" s="121"/>
+      <c r="Q28" s="107"/>
+      <c r="R28" s="108"/>
       <c r="S28" s="2"/>
     </row>
     <row r="29" spans="1:19" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="77" t="s">
         <v>77</v>
       </c>
-      <c r="B29" s="103" t="s">
+      <c r="B29" s="92" t="s">
         <v>76</v>
       </c>
-      <c r="C29" s="104"/>
+      <c r="C29" s="93"/>
       <c r="D29" s="51">
         <v>7</v>
       </c>
       <c r="E29" s="78"/>
-      <c r="F29" s="105">
+      <c r="F29" s="94">
         <v>46161</v>
       </c>
-      <c r="G29" s="106"/>
+      <c r="G29" s="95"/>
       <c r="H29" s="79">
         <v>0</v>
       </c>
-      <c r="I29" s="105">
+      <c r="I29" s="94">
         <v>46168</v>
       </c>
-      <c r="J29" s="106"/>
+      <c r="J29" s="95"/>
       <c r="K29" s="79"/>
       <c r="L29" s="54">
         <f t="shared" ref="L29" si="35">I29-F29</f>
         <v>7</v>
       </c>
-      <c r="M29" s="108">
+      <c r="M29" s="96">
         <f t="shared" si="28"/>
         <v>46175</v>
       </c>
-      <c r="N29" s="108"/>
+      <c r="N29" s="96"/>
       <c r="O29" s="55" t="str">
         <f t="shared" ref="O29" si="36">IFERROR(TEXT(WEEKDAY(M29),"ddd"),"")</f>
         <v>ter</v>
       </c>
       <c r="P29" s="29"/>
-      <c r="Q29" s="120"/>
-      <c r="R29" s="121"/>
+      <c r="Q29" s="107"/>
+      <c r="R29" s="108"/>
     </row>
     <row r="30" spans="1:19" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="100" t="s">
+      <c r="A30" s="109" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="101"/>
-      <c r="C30" s="102"/>
+      <c r="B30" s="110"/>
+      <c r="C30" s="111"/>
       <c r="D30" s="20" t="s">
         <v>15</v>
       </c>
       <c r="E30" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="F30" s="95" t="s">
+      <c r="F30" s="112" t="s">
         <v>18</v>
       </c>
-      <c r="G30" s="96"/>
-      <c r="H30" s="97"/>
-      <c r="I30" s="95" t="s">
+      <c r="G30" s="113"/>
+      <c r="H30" s="114"/>
+      <c r="I30" s="112" t="s">
         <v>17</v>
       </c>
-      <c r="J30" s="96"/>
-      <c r="K30" s="97"/>
+      <c r="J30" s="113"/>
+      <c r="K30" s="114"/>
       <c r="L30" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="M30" s="109" t="s">
+      <c r="M30" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="N30" s="110"/>
-      <c r="O30" s="111"/>
+      <c r="N30" s="116"/>
+      <c r="O30" s="117"/>
       <c r="P30" s="15" t="s">
         <v>11</v>
       </c>
@@ -2936,10 +2933,10 @@
       <c r="A31" s="17">
         <v>10</v>
       </c>
-      <c r="B31" s="122" t="s">
+      <c r="B31" s="100" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="123"/>
+      <c r="C31" s="101"/>
       <c r="D31" s="18">
         <v>7</v>
       </c>
@@ -3055,10 +3052,10 @@
     </row>
     <row r="34" spans="1:16" ht="21" x14ac:dyDescent="0.25">
       <c r="A34" s="27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B34" s="25" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C34" s="26"/>
       <c r="D34" s="18">
@@ -3169,7 +3166,7 @@
         <v>sex</v>
       </c>
       <c r="P36" s="19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3216,7 +3213,7 @@
         <v>1424</v>
       </c>
       <c r="B38" s="25" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C38" s="26"/>
       <c r="D38" s="18">
@@ -3286,7 +3283,7 @@
         <v>seg</v>
       </c>
       <c r="P39" s="19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="40" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3794,7 +3791,7 @@
         <v>qui</v>
       </c>
       <c r="P52" s="19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="53" spans="1:18" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3876,7 +3873,7 @@
         <v>ter</v>
       </c>
       <c r="P54" s="19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="55" spans="1:18" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -4041,10 +4038,10 @@
       <c r="A59" s="17">
         <v>109</v>
       </c>
-      <c r="B59" s="114" t="s">
+      <c r="B59" s="102" t="s">
         <v>42</v>
       </c>
-      <c r="C59" s="115"/>
+      <c r="C59" s="103"/>
       <c r="D59" s="18">
         <v>10</v>
       </c>
@@ -4075,12 +4072,12 @@
         <v>seg</v>
       </c>
       <c r="P59" s="19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="60" spans="1:18" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B60" s="25" t="s">
         <v>104</v>
@@ -4111,17 +4108,17 @@
       <c r="N60" s="91"/>
       <c r="O60" s="4"/>
       <c r="P60" s="19" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="61" spans="1:18" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="17">
         <v>110</v>
       </c>
-      <c r="B61" s="114" t="s">
+      <c r="B61" s="102" t="s">
         <v>43</v>
       </c>
-      <c r="C61" s="115"/>
+      <c r="C61" s="103"/>
       <c r="D61" s="18">
         <v>14</v>
       </c>
@@ -4154,17 +4151,17 @@
         <v>ter</v>
       </c>
       <c r="P61" s="19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="1:18" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="17">
         <v>1361</v>
       </c>
-      <c r="B62" s="114" t="s">
+      <c r="B62" s="102" t="s">
         <v>50</v>
       </c>
-      <c r="C62" s="115"/>
+      <c r="C62" s="103"/>
       <c r="D62" s="18">
         <v>25</v>
       </c>
@@ -4211,511 +4208,282 @@
       <c r="O63" s="8"/>
     </row>
     <row r="64" spans="1:18" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="93" t="str">
+      <c r="A64" s="118" t="str">
         <f>"Segunda(dia "&amp;TEXT($N$1+5,"DD")&amp;")"</f>
         <v>Segunda(dia 01)</v>
       </c>
-      <c r="B64" s="112"/>
-      <c r="C64" s="93" t="str">
+      <c r="B64" s="119"/>
+      <c r="C64" s="118" t="str">
         <f>"Terça(dia "&amp;TEXT($N$1+6,"DD")&amp;")"</f>
         <v>Terça(dia 02)</v>
       </c>
-      <c r="D64" s="112"/>
-      <c r="E64" s="112"/>
-      <c r="F64" s="94"/>
-      <c r="G64" s="112" t="str">
+      <c r="D64" s="119"/>
+      <c r="E64" s="119"/>
+      <c r="F64" s="121"/>
+      <c r="G64" s="119" t="str">
         <f>"Quarta(dia "&amp;TEXT($N$1+7,"DD")&amp;")"</f>
         <v>Quarta(dia 03)</v>
       </c>
-      <c r="H64" s="112"/>
-      <c r="I64" s="112"/>
-      <c r="J64" s="112"/>
-      <c r="K64" s="94"/>
-      <c r="L64" s="93" t="str">
+      <c r="H64" s="119"/>
+      <c r="I64" s="119"/>
+      <c r="J64" s="119"/>
+      <c r="K64" s="121"/>
+      <c r="L64" s="118" t="str">
         <f>"Quinta(dia "&amp;TEXT($N$1+8,"DD")&amp;")"</f>
         <v>Quinta(dia 04)</v>
       </c>
-      <c r="M64" s="112"/>
-      <c r="N64" s="112"/>
-      <c r="O64" s="112"/>
-      <c r="P64" s="94"/>
-      <c r="Q64" s="93" t="str">
+      <c r="M64" s="119"/>
+      <c r="N64" s="119"/>
+      <c r="O64" s="119"/>
+      <c r="P64" s="121"/>
+      <c r="Q64" s="118" t="str">
         <f>"Sexta(dia "&amp;TEXT($N$1+9,"DD")&amp;")"</f>
         <v>Sexta(dia 05)</v>
       </c>
-      <c r="R64" s="94"/>
+      <c r="R64" s="121"/>
     </row>
     <row r="65" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="88">
-        <v>1434</v>
-      </c>
-      <c r="B65" s="85" t="str">
-        <f t="shared" ref="B65:B83" si="78">IFERROR(VLOOKUP(A65,$A:$B,2,FALSE),"")</f>
-        <v>Hipermais - Araquari - Itinga</v>
-      </c>
-      <c r="C65" s="88">
-        <v>1435</v>
-      </c>
-      <c r="D65" s="92" t="str">
-        <f t="shared" ref="D65:D69" si="79">IFERROR(VLOOKUP(C65,$A:$B,2,FALSE),"")</f>
-        <v>Hipermais - Joinville - Vila Nova</v>
-      </c>
-      <c r="E65" s="92"/>
-      <c r="F65" s="92"/>
+      <c r="A65" s="88"/>
+      <c r="B65" s="85"/>
+      <c r="C65" s="88"/>
+      <c r="D65" s="106"/>
+      <c r="E65" s="106"/>
+      <c r="F65" s="106"/>
       <c r="G65" s="88"/>
-      <c r="H65" s="92" t="s">
-        <v>108</v>
-      </c>
-      <c r="I65" s="92"/>
-      <c r="J65" s="92"/>
-      <c r="K65" s="92"/>
-      <c r="L65" s="88">
-        <v>1346</v>
-      </c>
-      <c r="M65" s="92" t="str">
-        <f t="shared" ref="M65:M82" si="80">IFERROR(VLOOKUP(L65,$A:$B,2,FALSE),"")</f>
-        <v>Bistek Joinville - Aventureiro - Lj 09</v>
-      </c>
-      <c r="N65" s="92"/>
-      <c r="O65" s="92"/>
-      <c r="P65" s="92"/>
-      <c r="Q65" s="88">
-        <v>1437</v>
-      </c>
-      <c r="R65" s="92" t="str">
-        <f t="shared" ref="R65:R82" si="81">IFERROR(VLOOKUP(Q65,$A:$B,2,FALSE),"")</f>
-        <v>Hipermais - Jaraguá</v>
-      </c>
-      <c r="S65" s="92"/>
-      <c r="T65" s="92"/>
-      <c r="U65" s="92"/>
+      <c r="H65" s="106"/>
+      <c r="I65" s="106"/>
+      <c r="J65" s="106"/>
+      <c r="K65" s="106"/>
+      <c r="L65" s="88"/>
+      <c r="M65" s="106"/>
+      <c r="N65" s="106"/>
+      <c r="O65" s="106"/>
+      <c r="P65" s="106"/>
+      <c r="Q65" s="88"/>
+      <c r="R65" s="106"/>
+      <c r="S65" s="106"/>
+      <c r="T65" s="106"/>
+      <c r="U65" s="106"/>
     </row>
     <row r="66" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="88">
-        <v>1438</v>
-      </c>
-      <c r="B66" s="85" t="str">
-        <f t="shared" si="78"/>
-        <v>Hipermais CD - Joinville - Profipo</v>
-      </c>
-      <c r="C66" s="88">
-        <v>1429</v>
-      </c>
-      <c r="D66" s="92" t="str">
-        <f t="shared" si="79"/>
-        <v>Condor - America</v>
-      </c>
-      <c r="E66" s="92"/>
-      <c r="F66" s="92"/>
-      <c r="G66" s="88">
-        <v>1643</v>
-      </c>
-      <c r="H66" s="92" t="str">
-        <f t="shared" ref="H66:H82" si="82">IFERROR(VLOOKUP(G66,$A:$B,2,FALSE),"")</f>
-        <v>Hipermais - Joinville - Anita Garibaldi</v>
-      </c>
-      <c r="I66" s="92"/>
-      <c r="J66" s="92"/>
-      <c r="K66" s="92"/>
-      <c r="L66" s="88">
-        <v>1430</v>
-      </c>
-      <c r="M66" s="92" t="str">
-        <f t="shared" si="80"/>
-        <v>Condor - Boa Vista</v>
-      </c>
-      <c r="N66" s="92"/>
-      <c r="O66" s="92"/>
-      <c r="P66" s="92"/>
-      <c r="Q66" s="88">
-        <v>1425</v>
-      </c>
-      <c r="R66" s="85" t="str">
-        <f t="shared" si="81"/>
-        <v>Condor - Jaraguá</v>
-      </c>
+      <c r="A66" s="88"/>
+      <c r="B66" s="85"/>
+      <c r="C66" s="88"/>
+      <c r="D66" s="106"/>
+      <c r="E66" s="106"/>
+      <c r="F66" s="106"/>
+      <c r="G66" s="88"/>
+      <c r="H66" s="106"/>
+      <c r="I66" s="106"/>
+      <c r="J66" s="106"/>
+      <c r="K66" s="106"/>
+      <c r="L66" s="88"/>
+      <c r="M66" s="106"/>
+      <c r="N66" s="106"/>
+      <c r="O66" s="106"/>
+      <c r="P66" s="106"/>
+      <c r="Q66" s="88"/>
+      <c r="R66" s="85"/>
       <c r="S66" s="85"/>
       <c r="T66" s="85"/>
       <c r="U66" s="85"/>
     </row>
     <row r="67" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="88">
-        <v>1439</v>
-      </c>
-      <c r="B67" s="85" t="str">
-        <f t="shared" si="78"/>
-        <v>Hipermais - Joinville - Paranaguamirim</v>
-      </c>
-      <c r="C67" s="88">
-        <v>10</v>
-      </c>
-      <c r="D67" s="86" t="str">
-        <f t="shared" si="79"/>
-        <v>Angeloni - Joinville - América - Lj 21</v>
-      </c>
+      <c r="A67" s="88"/>
+      <c r="B67" s="85"/>
+      <c r="C67" s="88"/>
+      <c r="D67" s="86"/>
       <c r="E67" s="86"/>
       <c r="F67" s="86"/>
-      <c r="G67" s="88">
-        <v>1440</v>
-      </c>
-      <c r="H67" s="92" t="str">
-        <f t="shared" si="82"/>
-        <v>Hipermais - Joinville - João Costa</v>
-      </c>
-      <c r="I67" s="92"/>
-      <c r="J67" s="92"/>
-      <c r="K67" s="92"/>
-      <c r="L67" s="88">
-        <v>1429</v>
-      </c>
-      <c r="M67" s="92" t="str">
-        <f t="shared" si="80"/>
-        <v>Condor - America</v>
-      </c>
-      <c r="N67" s="92"/>
-      <c r="O67" s="92"/>
-      <c r="P67" s="92"/>
-      <c r="Q67" s="88">
-        <v>18</v>
-      </c>
-      <c r="R67" s="92" t="str">
-        <f t="shared" si="81"/>
-        <v>Angeloni - Jaraguá - Cel Grubba - Lj 22</v>
-      </c>
-      <c r="S67" s="92"/>
-      <c r="T67" s="92"/>
-      <c r="U67" s="92"/>
+      <c r="G67" s="88"/>
+      <c r="H67" s="106"/>
+      <c r="I67" s="106"/>
+      <c r="J67" s="106"/>
+      <c r="K67" s="106"/>
+      <c r="L67" s="88"/>
+      <c r="M67" s="106"/>
+      <c r="N67" s="106"/>
+      <c r="O67" s="106"/>
+      <c r="P67" s="106"/>
+      <c r="Q67" s="88"/>
+      <c r="R67" s="106"/>
+      <c r="S67" s="106"/>
+      <c r="T67" s="106"/>
+      <c r="U67" s="106"/>
     </row>
     <row r="68" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="88">
-        <v>1440</v>
-      </c>
-      <c r="B68" s="85" t="str">
-        <f t="shared" si="78"/>
-        <v>Hipermais - Joinville - João Costa</v>
-      </c>
-      <c r="C68" s="88" t="s">
-        <v>77</v>
-      </c>
-      <c r="D68" s="92" t="str">
-        <f t="shared" si="79"/>
-        <v>Fort - Penha - Lj 420</v>
-      </c>
-      <c r="E68" s="92"/>
-      <c r="F68" s="92"/>
-      <c r="G68" s="88" t="s">
-        <v>116</v>
-      </c>
-      <c r="H68" s="92" t="str">
-        <f t="shared" si="82"/>
-        <v>Angeloni - Joinville - centro - Lj 40</v>
-      </c>
-      <c r="I68" s="92"/>
-      <c r="J68" s="92"/>
-      <c r="K68" s="92"/>
-      <c r="L68" s="88">
-        <v>1436</v>
-      </c>
-      <c r="M68" s="92" t="str">
-        <f t="shared" si="80"/>
-        <v>Hipermais - Joinville - Fatima</v>
-      </c>
-      <c r="N68" s="92"/>
-      <c r="O68" s="92"/>
-      <c r="P68" s="92"/>
-      <c r="Q68" s="36" t="s">
-        <v>106</v>
-      </c>
-      <c r="R68" s="2" t="str">
-        <f t="shared" si="81"/>
-        <v xml:space="preserve">Brasil Atacadista - Itinga - Lj </v>
-      </c>
+      <c r="A68" s="88"/>
+      <c r="B68" s="85"/>
+      <c r="C68" s="88"/>
+      <c r="D68" s="106"/>
+      <c r="E68" s="106"/>
+      <c r="F68" s="106"/>
+      <c r="G68" s="88"/>
+      <c r="H68" s="106"/>
+      <c r="I68" s="106"/>
+      <c r="J68" s="106"/>
+      <c r="K68" s="106"/>
+      <c r="L68" s="88"/>
+      <c r="M68" s="106"/>
+      <c r="N68" s="106"/>
+      <c r="O68" s="106"/>
+      <c r="P68" s="106"/>
+      <c r="Q68" s="36"/>
+      <c r="R68" s="2"/>
     </row>
     <row r="69" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="88">
-        <v>1436</v>
-      </c>
-      <c r="B69" s="85" t="str">
-        <f t="shared" si="78"/>
-        <v>Hipermais - Joinville - Fatima</v>
-      </c>
-      <c r="C69" s="88" t="s">
-        <v>109</v>
-      </c>
-      <c r="D69" s="92" t="str">
-        <f t="shared" si="79"/>
-        <v>Fort - Barra Velha - Lj 335</v>
-      </c>
-      <c r="E69" s="92"/>
-      <c r="F69" s="92"/>
-      <c r="G69" s="36" t="s">
-        <v>54</v>
-      </c>
-      <c r="H69" s="107" t="str">
-        <f>IFERROR(VLOOKUP(G69,$A:$B,2,FALSE),"")</f>
-        <v>Condor - Itaum</v>
-      </c>
-      <c r="I69" s="107"/>
-      <c r="J69" s="107"/>
-      <c r="K69" s="107"/>
-      <c r="L69" s="88" t="s">
-        <v>26</v>
-      </c>
-      <c r="M69" s="92" t="str">
-        <f t="shared" si="80"/>
-        <v>Giassi - Joinville - América - Lj 08</v>
-      </c>
-      <c r="N69" s="92"/>
-      <c r="O69" s="92"/>
-      <c r="P69" s="92"/>
-      <c r="Q69" s="36" t="s">
-        <v>101</v>
-      </c>
-      <c r="R69" s="2" t="str">
-        <f t="shared" si="81"/>
-        <v>Dohler</v>
-      </c>
+      <c r="A69" s="88"/>
+      <c r="B69" s="85"/>
+      <c r="C69" s="88"/>
+      <c r="D69" s="106"/>
+      <c r="E69" s="106"/>
+      <c r="F69" s="106"/>
+      <c r="G69" s="36"/>
+      <c r="H69" s="105"/>
+      <c r="I69" s="105"/>
+      <c r="J69" s="105"/>
+      <c r="K69" s="105"/>
+      <c r="L69" s="88"/>
+      <c r="M69" s="106"/>
+      <c r="N69" s="106"/>
+      <c r="O69" s="106"/>
+      <c r="P69" s="106"/>
+      <c r="Q69" s="36"/>
+      <c r="R69" s="2"/>
     </row>
     <row r="70" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="88">
-        <v>1424</v>
-      </c>
-      <c r="B70" s="85" t="str">
-        <f t="shared" si="78"/>
-        <v xml:space="preserve">Condor  - Itaum </v>
-      </c>
-      <c r="C70" s="88">
-        <v>1605</v>
-      </c>
-      <c r="D70" s="92" t="str">
-        <f t="shared" ref="D70:D78" si="83">IFERROR(VLOOKUP(C70,$A:$B,2,FALSE),"")</f>
-        <v>Fort - Joinville - Vila Nova</v>
-      </c>
-      <c r="E70" s="92"/>
-      <c r="F70" s="92"/>
-      <c r="G70" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="H70" s="107" t="str">
-        <f t="shared" ref="H70:H78" si="84">IFERROR(VLOOKUP(G70,$A:$B,2,FALSE),"")</f>
-        <v>Fort - Joinville - Floresta - Lj 250</v>
-      </c>
-      <c r="I70" s="107"/>
-      <c r="J70" s="107"/>
-      <c r="K70" s="107"/>
-      <c r="L70" s="88" t="s">
-        <v>29</v>
-      </c>
-      <c r="M70" s="92" t="str">
-        <f t="shared" si="80"/>
-        <v>Giassi - Joinville - América - Lj 08</v>
-      </c>
-      <c r="N70" s="92"/>
-      <c r="O70" s="92"/>
-      <c r="P70" s="92"/>
-      <c r="Q70" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="R70" s="2" t="str">
-        <f t="shared" si="81"/>
-        <v>Giassi - Jaraguá - Centro - Lj 15</v>
-      </c>
+      <c r="A70" s="88"/>
+      <c r="B70" s="85"/>
+      <c r="C70" s="88"/>
+      <c r="D70" s="106"/>
+      <c r="E70" s="106"/>
+      <c r="F70" s="106"/>
+      <c r="G70" s="36"/>
+      <c r="H70" s="105"/>
+      <c r="I70" s="105"/>
+      <c r="J70" s="105"/>
+      <c r="K70" s="105"/>
+      <c r="L70" s="88"/>
+      <c r="M70" s="106"/>
+      <c r="N70" s="106"/>
+      <c r="O70" s="106"/>
+      <c r="P70" s="106"/>
+      <c r="Q70" s="36"/>
+      <c r="R70" s="2"/>
       <c r="S70" s="35"/>
-      <c r="T70" s="83" t="str">
-        <f>IFERROR(VLOOKUP(S70,$A:$B,2,FALSE),"")</f>
-        <v/>
-      </c>
     </row>
     <row r="71" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="88" t="s">
-        <v>60</v>
-      </c>
-      <c r="B71" s="85" t="str">
-        <f t="shared" si="78"/>
-        <v>Giassi - Joinville LJ 08</v>
-      </c>
-      <c r="C71" s="36" t="s">
-        <v>75</v>
-      </c>
-      <c r="D71" s="119" t="str">
-        <f t="shared" si="83"/>
-        <v>Fort - Penha - Lj 420</v>
-      </c>
-      <c r="E71" s="119"/>
-      <c r="F71" s="119"/>
+      <c r="A71" s="88"/>
+      <c r="B71" s="85"/>
+      <c r="C71" s="36"/>
+      <c r="D71" s="104"/>
+      <c r="E71" s="104"/>
+      <c r="F71" s="104"/>
       <c r="G71" s="36"/>
-      <c r="H71" s="107" t="str">
-        <f t="shared" si="84"/>
-        <v/>
-      </c>
-      <c r="I71" s="107"/>
-      <c r="J71" s="107"/>
-      <c r="K71" s="107"/>
-      <c r="L71" s="88" t="s">
-        <v>32</v>
-      </c>
-      <c r="M71" s="92" t="str">
-        <f t="shared" si="80"/>
-        <v>Fort - Joinville - Aventureiro - Lj 165</v>
-      </c>
-      <c r="N71" s="92"/>
-      <c r="O71" s="92"/>
-      <c r="P71" s="92"/>
-      <c r="Q71" s="36" t="s">
-        <v>30</v>
-      </c>
-      <c r="R71" s="2" t="str">
-        <f t="shared" si="81"/>
-        <v>Giassi - Joinville - Bucarein - Lj 14</v>
-      </c>
+      <c r="H71" s="105"/>
+      <c r="I71" s="105"/>
+      <c r="J71" s="105"/>
+      <c r="K71" s="105"/>
+      <c r="L71" s="88"/>
+      <c r="M71" s="106"/>
+      <c r="N71" s="106"/>
+      <c r="O71" s="106"/>
+      <c r="P71" s="106"/>
+      <c r="Q71" s="36"/>
+      <c r="R71" s="2"/>
     </row>
     <row r="72" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="88" t="s">
-        <v>29</v>
-      </c>
-      <c r="B72" s="85" t="str">
-        <f t="shared" si="78"/>
-        <v>Giassi - Joinville - América - Lj 08</v>
-      </c>
-      <c r="C72" s="36" t="s">
-        <v>48</v>
-      </c>
-      <c r="D72" s="119" t="str">
-        <f t="shared" ref="D72" si="85">IFERROR(VLOOKUP(C72,$A:$B,2,FALSE),"")</f>
-        <v>Benteler</v>
-      </c>
-      <c r="E72" s="119"/>
-      <c r="F72" s="119"/>
+      <c r="A72" s="88"/>
+      <c r="B72" s="85"/>
+      <c r="C72" s="36"/>
+      <c r="D72" s="104"/>
+      <c r="E72" s="104"/>
+      <c r="F72" s="104"/>
       <c r="G72" s="36"/>
-      <c r="H72" s="107" t="str">
-        <f t="shared" si="84"/>
-        <v/>
-      </c>
-      <c r="I72" s="107"/>
-      <c r="J72" s="107"/>
-      <c r="K72" s="107"/>
+      <c r="H72" s="105"/>
+      <c r="I72" s="105"/>
+      <c r="J72" s="105"/>
+      <c r="K72" s="105"/>
       <c r="L72" s="36"/>
-      <c r="M72" s="107" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N72" s="107"/>
-      <c r="O72" s="107"/>
-      <c r="P72" s="107"/>
-      <c r="Q72" s="36" t="s">
-        <v>120</v>
-      </c>
-      <c r="R72" s="2" t="str">
-        <f t="shared" si="81"/>
-        <v>Fort São Francisco do Sul - Lj 395</v>
-      </c>
+      <c r="M72" s="105"/>
+      <c r="N72" s="105"/>
+      <c r="O72" s="105"/>
+      <c r="P72" s="105"/>
+      <c r="Q72" s="36"/>
+      <c r="R72" s="2"/>
     </row>
     <row r="73" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="36" t="s">
-        <v>23</v>
-      </c>
-      <c r="B73" s="2" t="str">
-        <f t="shared" si="78"/>
-        <v>Fort - Joinville - Aventureiro - Lj 165</v>
-      </c>
+      <c r="A73" s="36"/>
+      <c r="B73" s="2"/>
       <c r="C73" s="36"/>
-      <c r="D73" s="119" t="str">
-        <f t="shared" si="83"/>
-        <v/>
-      </c>
-      <c r="E73" s="119"/>
-      <c r="F73" s="119"/>
+      <c r="D73" s="104"/>
+      <c r="E73" s="104"/>
+      <c r="F73" s="104"/>
       <c r="G73" s="36"/>
-      <c r="H73" s="107" t="str">
-        <f t="shared" si="84"/>
-        <v/>
-      </c>
-      <c r="I73" s="107"/>
-      <c r="J73" s="107"/>
-      <c r="K73" s="107"/>
+      <c r="H73" s="105"/>
+      <c r="I73" s="105"/>
+      <c r="J73" s="105"/>
+      <c r="K73" s="105"/>
       <c r="L73" s="36"/>
-      <c r="M73" s="119" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N73" s="119"/>
-      <c r="O73" s="119"/>
-      <c r="P73" s="119"/>
+      <c r="M73" s="104"/>
+      <c r="N73" s="104"/>
+      <c r="O73" s="104"/>
+      <c r="P73" s="104"/>
       <c r="Q73" s="36"/>
-      <c r="R73" s="2" t="str">
-        <f t="shared" si="81"/>
-        <v/>
-      </c>
+      <c r="R73" s="2"/>
     </row>
     <row r="74" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="36" t="s">
-        <v>30</v>
-      </c>
-      <c r="B74" s="2" t="str">
-        <f t="shared" si="78"/>
-        <v>Giassi - Joinville - Bucarein - Lj 14</v>
-      </c>
+      <c r="A74" s="36"/>
+      <c r="B74" s="2"/>
       <c r="C74" s="36"/>
-      <c r="D74" s="119" t="str">
-        <f t="shared" si="83"/>
-        <v/>
-      </c>
-      <c r="E74" s="119"/>
-      <c r="F74" s="119"/>
+      <c r="D74" s="104"/>
+      <c r="E74" s="104"/>
+      <c r="F74" s="104"/>
       <c r="G74" s="36"/>
-      <c r="H74" s="107" t="str">
-        <f t="shared" si="84"/>
-        <v/>
-      </c>
-      <c r="I74" s="107"/>
-      <c r="J74" s="107"/>
-      <c r="K74" s="107"/>
+      <c r="H74" s="105"/>
+      <c r="I74" s="105"/>
+      <c r="J74" s="105"/>
+      <c r="K74" s="105"/>
       <c r="L74" s="36"/>
-      <c r="M74" s="119" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N74" s="119"/>
-      <c r="O74" s="119"/>
-      <c r="P74" s="119"/>
+      <c r="M74" s="104"/>
+      <c r="N74" s="104"/>
+      <c r="O74" s="104"/>
+      <c r="P74" s="104"/>
       <c r="Q74" s="36"/>
-      <c r="R74" s="2" t="str">
-        <f t="shared" si="81"/>
-        <v/>
-      </c>
+      <c r="R74" s="2"/>
     </row>
     <row r="75" spans="1:21" s="83" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="36"/>
       <c r="B75" s="2" t="str">
-        <f t="shared" si="78"/>
+        <f t="shared" ref="B65:B83" si="78">IFERROR(VLOOKUP(A75,$A:$B,2,FALSE),"")</f>
         <v/>
       </c>
       <c r="C75" s="36"/>
-      <c r="D75" s="119" t="str">
-        <f t="shared" si="83"/>
-        <v/>
-      </c>
-      <c r="E75" s="119"/>
-      <c r="F75" s="119"/>
+      <c r="D75" s="104" t="str">
+        <f t="shared" ref="D70:D78" si="79">IFERROR(VLOOKUP(C75,$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="E75" s="104"/>
+      <c r="F75" s="104"/>
       <c r="G75" s="36"/>
-      <c r="H75" s="107" t="str">
-        <f t="shared" si="84"/>
-        <v/>
-      </c>
-      <c r="I75" s="107"/>
-      <c r="J75" s="107"/>
-      <c r="K75" s="107"/>
+      <c r="H75" s="105" t="str">
+        <f t="shared" ref="H70:H78" si="80">IFERROR(VLOOKUP(G75,$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I75" s="105"/>
+      <c r="J75" s="105"/>
+      <c r="K75" s="105"/>
       <c r="L75" s="36"/>
-      <c r="M75" s="119" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N75" s="119"/>
-      <c r="O75" s="119"/>
-      <c r="P75" s="119"/>
+      <c r="M75" s="104" t="str">
+        <f t="shared" ref="M65:M82" si="81">IFERROR(VLOOKUP(L75,$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="N75" s="104"/>
+      <c r="O75" s="104"/>
+      <c r="P75" s="104"/>
       <c r="Q75" s="36"/>
       <c r="R75" s="2" t="str">
-        <f t="shared" si="81"/>
+        <f t="shared" ref="R65:R82" si="82">IFERROR(VLOOKUP(Q75,$A:$B,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
@@ -4726,31 +4494,31 @@
         <v/>
       </c>
       <c r="C76" s="36"/>
-      <c r="D76" s="119" t="str">
-        <f t="shared" si="83"/>
-        <v/>
-      </c>
-      <c r="E76" s="119"/>
-      <c r="F76" s="119"/>
+      <c r="D76" s="104" t="str">
+        <f t="shared" si="79"/>
+        <v/>
+      </c>
+      <c r="E76" s="104"/>
+      <c r="F76" s="104"/>
       <c r="G76" s="36"/>
-      <c r="H76" s="107" t="str">
-        <f t="shared" si="84"/>
-        <v/>
-      </c>
-      <c r="I76" s="107"/>
-      <c r="J76" s="107"/>
-      <c r="K76" s="107"/>
+      <c r="H76" s="105" t="str">
+        <f t="shared" si="80"/>
+        <v/>
+      </c>
+      <c r="I76" s="105"/>
+      <c r="J76" s="105"/>
+      <c r="K76" s="105"/>
       <c r="L76" s="36"/>
-      <c r="M76" s="119" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N76" s="119"/>
-      <c r="O76" s="119"/>
-      <c r="P76" s="119"/>
+      <c r="M76" s="104" t="str">
+        <f t="shared" si="81"/>
+        <v/>
+      </c>
+      <c r="N76" s="104"/>
+      <c r="O76" s="104"/>
+      <c r="P76" s="104"/>
       <c r="Q76" s="37"/>
       <c r="R76" s="2" t="str">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v/>
       </c>
     </row>
@@ -4761,31 +4529,31 @@
         <v/>
       </c>
       <c r="C77" s="36"/>
-      <c r="D77" s="119" t="str">
-        <f t="shared" si="83"/>
-        <v/>
-      </c>
-      <c r="E77" s="119"/>
-      <c r="F77" s="119"/>
+      <c r="D77" s="104" t="str">
+        <f t="shared" si="79"/>
+        <v/>
+      </c>
+      <c r="E77" s="104"/>
+      <c r="F77" s="104"/>
       <c r="G77" s="36"/>
-      <c r="H77" s="107" t="str">
-        <f t="shared" si="84"/>
-        <v/>
-      </c>
-      <c r="I77" s="107"/>
-      <c r="J77" s="107"/>
-      <c r="K77" s="107"/>
+      <c r="H77" s="105" t="str">
+        <f t="shared" si="80"/>
+        <v/>
+      </c>
+      <c r="I77" s="105"/>
+      <c r="J77" s="105"/>
+      <c r="K77" s="105"/>
       <c r="L77" s="38"/>
-      <c r="M77" s="119" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N77" s="119"/>
-      <c r="O77" s="119"/>
-      <c r="P77" s="119"/>
+      <c r="M77" s="104" t="str">
+        <f t="shared" si="81"/>
+        <v/>
+      </c>
+      <c r="N77" s="104"/>
+      <c r="O77" s="104"/>
+      <c r="P77" s="104"/>
       <c r="Q77" s="37"/>
       <c r="R77" s="2" t="str">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v/>
       </c>
     </row>
@@ -4796,62 +4564,62 @@
         <v/>
       </c>
       <c r="C78" s="37"/>
-      <c r="D78" s="119" t="str">
-        <f t="shared" si="83"/>
-        <v/>
-      </c>
-      <c r="E78" s="119"/>
-      <c r="F78" s="119"/>
+      <c r="D78" s="104" t="str">
+        <f t="shared" si="79"/>
+        <v/>
+      </c>
+      <c r="E78" s="104"/>
+      <c r="F78" s="104"/>
       <c r="G78" s="36"/>
-      <c r="H78" s="107" t="str">
-        <f t="shared" si="84"/>
-        <v/>
-      </c>
-      <c r="I78" s="107"/>
-      <c r="J78" s="107"/>
-      <c r="K78" s="107"/>
+      <c r="H78" s="105" t="str">
+        <f t="shared" si="80"/>
+        <v/>
+      </c>
+      <c r="I78" s="105"/>
+      <c r="J78" s="105"/>
+      <c r="K78" s="105"/>
       <c r="L78" s="38"/>
-      <c r="M78" s="119" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N78" s="119"/>
-      <c r="O78" s="119"/>
-      <c r="P78" s="119"/>
+      <c r="M78" s="104" t="str">
+        <f t="shared" si="81"/>
+        <v/>
+      </c>
+      <c r="N78" s="104"/>
+      <c r="O78" s="104"/>
+      <c r="P78" s="104"/>
       <c r="Q78" s="37"/>
       <c r="R78" s="2" t="str">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v/>
       </c>
     </row>
     <row r="79" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="36"/>
       <c r="C79" s="37"/>
-      <c r="D79" s="119" t="str">
-        <f t="shared" ref="D79:D80" si="86">IFERROR(VLOOKUP(C79,$A:$B,2,FALSE),"")</f>
-        <v/>
-      </c>
-      <c r="E79" s="119"/>
-      <c r="F79" s="119"/>
+      <c r="D79" s="104" t="str">
+        <f t="shared" ref="D79:D80" si="83">IFERROR(VLOOKUP(C79,$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="E79" s="104"/>
+      <c r="F79" s="104"/>
       <c r="G79" s="36"/>
-      <c r="H79" s="119" t="str">
-        <f t="shared" si="82"/>
-        <v/>
-      </c>
-      <c r="I79" s="119"/>
-      <c r="J79" s="119"/>
-      <c r="K79" s="119"/>
+      <c r="H79" s="104" t="str">
+        <f t="shared" ref="H66:H82" si="84">IFERROR(VLOOKUP(G79,$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="I79" s="104"/>
+      <c r="J79" s="104"/>
+      <c r="K79" s="104"/>
       <c r="L79" s="38"/>
-      <c r="M79" s="119" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N79" s="119"/>
-      <c r="O79" s="119"/>
-      <c r="P79" s="119"/>
+      <c r="M79" s="104" t="str">
+        <f t="shared" si="81"/>
+        <v/>
+      </c>
+      <c r="N79" s="104"/>
+      <c r="O79" s="104"/>
+      <c r="P79" s="104"/>
       <c r="Q79" s="37"/>
       <c r="R79" s="2" t="str">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v/>
       </c>
     </row>
@@ -4861,31 +4629,31 @@
         <v/>
       </c>
       <c r="C80" s="37"/>
-      <c r="D80" s="119" t="str">
-        <f t="shared" si="86"/>
-        <v/>
-      </c>
-      <c r="E80" s="119"/>
-      <c r="F80" s="119"/>
+      <c r="D80" s="104" t="str">
+        <f t="shared" si="83"/>
+        <v/>
+      </c>
+      <c r="E80" s="104"/>
+      <c r="F80" s="104"/>
       <c r="G80" s="36"/>
-      <c r="H80" s="119" t="str">
-        <f t="shared" si="82"/>
-        <v/>
-      </c>
-      <c r="I80" s="119"/>
-      <c r="J80" s="119"/>
-      <c r="K80" s="119"/>
+      <c r="H80" s="104" t="str">
+        <f t="shared" si="84"/>
+        <v/>
+      </c>
+      <c r="I80" s="104"/>
+      <c r="J80" s="104"/>
+      <c r="K80" s="104"/>
       <c r="L80" s="38"/>
-      <c r="M80" s="119" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N80" s="119"/>
-      <c r="O80" s="119"/>
-      <c r="P80" s="119"/>
+      <c r="M80" s="104" t="str">
+        <f t="shared" si="81"/>
+        <v/>
+      </c>
+      <c r="N80" s="104"/>
+      <c r="O80" s="104"/>
+      <c r="P80" s="104"/>
       <c r="Q80" s="37"/>
       <c r="R80" s="2" t="str">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v/>
       </c>
     </row>
@@ -4896,31 +4664,31 @@
         <v/>
       </c>
       <c r="C81" s="37"/>
-      <c r="D81" s="119" t="str">
-        <f t="shared" ref="D81:D82" si="87">IFERROR(VLOOKUP(C81,$A:$B,2,FALSE),"")</f>
-        <v/>
-      </c>
-      <c r="E81" s="119"/>
-      <c r="F81" s="119"/>
+      <c r="D81" s="104" t="str">
+        <f t="shared" ref="D81:D82" si="85">IFERROR(VLOOKUP(C81,$A:$B,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="E81" s="104"/>
+      <c r="F81" s="104"/>
       <c r="G81" s="36"/>
-      <c r="H81" s="119" t="str">
-        <f t="shared" si="82"/>
-        <v/>
-      </c>
-      <c r="I81" s="119"/>
-      <c r="J81" s="119"/>
-      <c r="K81" s="119"/>
+      <c r="H81" s="104" t="str">
+        <f t="shared" si="84"/>
+        <v/>
+      </c>
+      <c r="I81" s="104"/>
+      <c r="J81" s="104"/>
+      <c r="K81" s="104"/>
       <c r="L81" s="38"/>
-      <c r="M81" s="119" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N81" s="119"/>
-      <c r="O81" s="119"/>
-      <c r="P81" s="119"/>
+      <c r="M81" s="104" t="str">
+        <f t="shared" si="81"/>
+        <v/>
+      </c>
+      <c r="N81" s="104"/>
+      <c r="O81" s="104"/>
+      <c r="P81" s="104"/>
       <c r="Q81" s="37"/>
       <c r="R81" s="2" t="str">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v/>
       </c>
     </row>
@@ -4931,31 +4699,31 @@
         <v/>
       </c>
       <c r="C82" s="37"/>
-      <c r="D82" s="119" t="str">
-        <f t="shared" si="87"/>
-        <v/>
-      </c>
-      <c r="E82" s="119"/>
-      <c r="F82" s="119"/>
+      <c r="D82" s="104" t="str">
+        <f t="shared" si="85"/>
+        <v/>
+      </c>
+      <c r="E82" s="104"/>
+      <c r="F82" s="104"/>
       <c r="G82" s="36"/>
-      <c r="H82" s="119" t="str">
-        <f t="shared" si="82"/>
-        <v/>
-      </c>
-      <c r="I82" s="119"/>
-      <c r="J82" s="119"/>
-      <c r="K82" s="119"/>
+      <c r="H82" s="104" t="str">
+        <f t="shared" si="84"/>
+        <v/>
+      </c>
+      <c r="I82" s="104"/>
+      <c r="J82" s="104"/>
+      <c r="K82" s="104"/>
       <c r="L82" s="38"/>
-      <c r="M82" s="119" t="str">
-        <f t="shared" si="80"/>
-        <v/>
-      </c>
-      <c r="N82" s="119"/>
-      <c r="O82" s="119"/>
-      <c r="P82" s="119"/>
+      <c r="M82" s="104" t="str">
+        <f t="shared" si="81"/>
+        <v/>
+      </c>
+      <c r="N82" s="104"/>
+      <c r="O82" s="104"/>
+      <c r="P82" s="104"/>
       <c r="Q82" s="37"/>
       <c r="R82" s="2" t="str">
-        <f t="shared" si="81"/>
+        <f t="shared" si="82"/>
         <v/>
       </c>
     </row>
@@ -5020,6 +4788,241 @@
     <filterColumn colId="13" showButton="0"/>
   </autoFilter>
   <mergeCells count="259">
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="M51:N51"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="M44:N44"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="M48:N48"/>
+    <mergeCell ref="M46:N46"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="M47:N47"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="M43:N43"/>
+    <mergeCell ref="M41:N41"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="M61:N61"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="I54:J54"/>
+    <mergeCell ref="M54:N54"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="M59:N59"/>
+    <mergeCell ref="F57:G57"/>
+    <mergeCell ref="I57:J57"/>
+    <mergeCell ref="M57:N57"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="I52:J52"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="M42:N42"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="M45:N45"/>
+    <mergeCell ref="M52:N52"/>
+    <mergeCell ref="R67:U67"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="M49:N49"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="M50:N50"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="I56:J56"/>
+    <mergeCell ref="M56:N56"/>
+    <mergeCell ref="H67:K67"/>
+    <mergeCell ref="R65:U65"/>
+    <mergeCell ref="D66:F66"/>
+    <mergeCell ref="H66:K66"/>
+    <mergeCell ref="M66:P66"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="M53:N53"/>
+    <mergeCell ref="Q64:R64"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="H65:K65"/>
+    <mergeCell ref="M65:P65"/>
+    <mergeCell ref="I55:J55"/>
+    <mergeCell ref="M55:N55"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H69:K69"/>
+    <mergeCell ref="M69:P69"/>
+    <mergeCell ref="M67:P67"/>
+    <mergeCell ref="M68:P68"/>
+    <mergeCell ref="H68:K68"/>
+    <mergeCell ref="D68:F68"/>
+    <mergeCell ref="M40:N40"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="M36:N36"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="M39:N39"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="M30:O30"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="I62:J62"/>
+    <mergeCell ref="M62:N62"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="F58:G58"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C64:F64"/>
+    <mergeCell ref="G64:K64"/>
+    <mergeCell ref="L64:P64"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="M2:O2"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="D69:F69"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="D82:F82"/>
+    <mergeCell ref="H82:K82"/>
+    <mergeCell ref="M82:P82"/>
+    <mergeCell ref="D76:F76"/>
+    <mergeCell ref="D81:F81"/>
+    <mergeCell ref="H81:K81"/>
+    <mergeCell ref="M81:P81"/>
+    <mergeCell ref="D78:F78"/>
+    <mergeCell ref="H78:K78"/>
+    <mergeCell ref="M78:P78"/>
+    <mergeCell ref="D79:F79"/>
+    <mergeCell ref="H79:K79"/>
+    <mergeCell ref="M79:P79"/>
+    <mergeCell ref="D80:F80"/>
+    <mergeCell ref="H80:K80"/>
+    <mergeCell ref="M80:P80"/>
+    <mergeCell ref="H70:K70"/>
+    <mergeCell ref="D77:F77"/>
+    <mergeCell ref="H77:K77"/>
+    <mergeCell ref="Q21:R29"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="D71:F71"/>
+    <mergeCell ref="M72:P72"/>
+    <mergeCell ref="D73:F73"/>
+    <mergeCell ref="M73:P73"/>
+    <mergeCell ref="H72:K72"/>
+    <mergeCell ref="H73:K73"/>
+    <mergeCell ref="M70:P70"/>
+    <mergeCell ref="H71:K71"/>
+    <mergeCell ref="M71:P71"/>
+    <mergeCell ref="D70:F70"/>
+    <mergeCell ref="D72:F72"/>
+    <mergeCell ref="M77:P77"/>
+    <mergeCell ref="D74:F74"/>
+    <mergeCell ref="H76:K76"/>
+    <mergeCell ref="M76:P76"/>
+    <mergeCell ref="H74:K74"/>
+    <mergeCell ref="M74:P74"/>
+    <mergeCell ref="D75:F75"/>
+    <mergeCell ref="H75:K75"/>
+    <mergeCell ref="M75:P75"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="M15:N15"/>
     <mergeCell ref="F60:G60"/>
     <mergeCell ref="I60:J60"/>
     <mergeCell ref="M60:N60"/>
@@ -5044,243 +5047,8 @@
     <mergeCell ref="I27:J27"/>
     <mergeCell ref="M27:N27"/>
     <mergeCell ref="I40:J40"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M77:P77"/>
-    <mergeCell ref="D74:F74"/>
-    <mergeCell ref="H76:K76"/>
-    <mergeCell ref="M76:P76"/>
-    <mergeCell ref="H74:K74"/>
-    <mergeCell ref="M74:P74"/>
-    <mergeCell ref="D75:F75"/>
-    <mergeCell ref="H75:K75"/>
-    <mergeCell ref="M75:P75"/>
-    <mergeCell ref="D71:F71"/>
-    <mergeCell ref="M72:P72"/>
-    <mergeCell ref="D73:F73"/>
-    <mergeCell ref="M73:P73"/>
-    <mergeCell ref="H72:K72"/>
-    <mergeCell ref="H73:K73"/>
-    <mergeCell ref="M70:P70"/>
-    <mergeCell ref="H71:K71"/>
-    <mergeCell ref="M71:P71"/>
-    <mergeCell ref="D70:F70"/>
-    <mergeCell ref="D72:F72"/>
-    <mergeCell ref="Q21:R29"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="F61:G61"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="D69:F69"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="D82:F82"/>
-    <mergeCell ref="H82:K82"/>
-    <mergeCell ref="M82:P82"/>
-    <mergeCell ref="D76:F76"/>
-    <mergeCell ref="D81:F81"/>
-    <mergeCell ref="H81:K81"/>
-    <mergeCell ref="M81:P81"/>
-    <mergeCell ref="D78:F78"/>
-    <mergeCell ref="H78:K78"/>
-    <mergeCell ref="M78:P78"/>
-    <mergeCell ref="D79:F79"/>
-    <mergeCell ref="H79:K79"/>
-    <mergeCell ref="M79:P79"/>
-    <mergeCell ref="D80:F80"/>
-    <mergeCell ref="H80:K80"/>
-    <mergeCell ref="M80:P80"/>
-    <mergeCell ref="H70:K70"/>
-    <mergeCell ref="D77:F77"/>
-    <mergeCell ref="H77:K77"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="M2:O2"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="M10:N10"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="A64:B64"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="I62:J62"/>
-    <mergeCell ref="M62:N62"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="F58:G58"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="C64:F64"/>
-    <mergeCell ref="G64:K64"/>
-    <mergeCell ref="L64:P64"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="H69:K69"/>
-    <mergeCell ref="M69:P69"/>
-    <mergeCell ref="M67:P67"/>
-    <mergeCell ref="M68:P68"/>
-    <mergeCell ref="H68:K68"/>
-    <mergeCell ref="D68:F68"/>
-    <mergeCell ref="M40:N40"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="M39:N39"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="M30:O30"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="R67:U67"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="M49:N49"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="M50:N50"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="I56:J56"/>
-    <mergeCell ref="M56:N56"/>
-    <mergeCell ref="H67:K67"/>
-    <mergeCell ref="R65:U65"/>
-    <mergeCell ref="D66:F66"/>
-    <mergeCell ref="H66:K66"/>
-    <mergeCell ref="M66:P66"/>
-    <mergeCell ref="I53:J53"/>
-    <mergeCell ref="M53:N53"/>
-    <mergeCell ref="Q64:R64"/>
-    <mergeCell ref="D65:F65"/>
-    <mergeCell ref="H65:K65"/>
-    <mergeCell ref="M65:P65"/>
-    <mergeCell ref="I55:J55"/>
-    <mergeCell ref="M55:N55"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="M43:N43"/>
-    <mergeCell ref="M41:N41"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="M61:N61"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="I54:J54"/>
-    <mergeCell ref="M54:N54"/>
-    <mergeCell ref="F55:G55"/>
-    <mergeCell ref="M59:N59"/>
-    <mergeCell ref="F57:G57"/>
-    <mergeCell ref="I57:J57"/>
-    <mergeCell ref="M57:N57"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="I52:J52"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="M42:N42"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="M45:N45"/>
-    <mergeCell ref="M52:N52"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="M51:N51"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="M48:N48"/>
-    <mergeCell ref="M46:N46"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="M47:N47"/>
-    <mergeCell ref="F46:G46"/>
   </mergeCells>
-  <conditionalFormatting sqref="M31:O62 M3:O29">
+  <conditionalFormatting sqref="M3:O29 M31:O62">
     <cfRule type="expression" dxfId="7" priority="176">
       <formula>IF(IFERROR(VLOOKUP($A3,$A$64:$A$83,1,FALSE),"")&amp;IFERROR(VLOOKUP($A3,$C$64:$C$83,1,FALSE),"")&amp;IFERROR(VLOOKUP($A3,$G$64:$G$83,1,FALSE),"")&amp;IFERROR(VLOOKUP($A3,$L$64:$L$83,1,FALSE),"")&amp;IFERROR(VLOOKUP($A3,$Q$64:$Q$83,1,FALSE),"")="",FALSE(),TRUE())</formula>
     </cfRule>
@@ -5351,41 +5119,41 @@
       <c r="M1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="113">
+      <c r="N1" s="120">
         <v>45819</v>
       </c>
-      <c r="O1" s="113"/>
+      <c r="O1" s="120"/>
     </row>
     <row r="2" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="100" t="s">
+      <c r="A2" s="109" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="101"/>
-      <c r="C2" s="102"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="111"/>
       <c r="D2" s="20" t="s">
         <v>15</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="95" t="s">
+      <c r="F2" s="112" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="96"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="95" t="s">
+      <c r="G2" s="113"/>
+      <c r="H2" s="114"/>
+      <c r="I2" s="112" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="96"/>
-      <c r="K2" s="97"/>
+      <c r="J2" s="113"/>
+      <c r="K2" s="114"/>
       <c r="L2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="109" t="s">
+      <c r="M2" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="N2" s="110"/>
-      <c r="O2" s="111"/>
+      <c r="N2" s="116"/>
+      <c r="O2" s="117"/>
       <c r="P2" s="15" t="s">
         <v>81</v>
       </c>
@@ -5521,17 +5289,17 @@
         <v>20</v>
       </c>
       <c r="E6" s="52"/>
-      <c r="F6" s="105">
+      <c r="F6" s="94">
         <v>45786</v>
       </c>
-      <c r="G6" s="106"/>
+      <c r="G6" s="95"/>
       <c r="H6" s="53">
         <v>5490</v>
       </c>
-      <c r="I6" s="105">
+      <c r="I6" s="94">
         <v>45807</v>
       </c>
-      <c r="J6" s="106"/>
+      <c r="J6" s="95"/>
       <c r="K6" s="53">
         <v>6460</v>
       </c>
@@ -5539,11 +5307,11 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="M6" s="108">
+      <c r="M6" s="96">
         <f t="shared" si="1"/>
         <v>45827</v>
       </c>
-      <c r="N6" s="108"/>
+      <c r="N6" s="96"/>
       <c r="O6" s="55" t="str">
         <f t="shared" si="2"/>
         <v>qui</v>
@@ -5710,10 +5478,10 @@
       <c r="A11" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="114" t="s">
+      <c r="B11" s="102" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="114"/>
+      <c r="C11" s="102"/>
       <c r="D11" s="30">
         <v>20</v>
       </c>
@@ -5821,10 +5589,10 @@
       <c r="A14" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="114" t="s">
+      <c r="B14" s="102" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="115"/>
+      <c r="C14" s="103"/>
       <c r="D14" s="30">
         <v>9</v>
       </c>
@@ -5905,34 +5673,34 @@
         <v>15</v>
       </c>
       <c r="E16" s="61"/>
-      <c r="F16" s="132">
+      <c r="F16" s="126">
         <v>45793</v>
       </c>
-      <c r="G16" s="133"/>
+      <c r="G16" s="127"/>
       <c r="H16" s="62"/>
-      <c r="I16" s="132">
+      <c r="I16" s="126">
         <v>45805</v>
       </c>
-      <c r="J16" s="133"/>
+      <c r="J16" s="127"/>
       <c r="K16" s="62"/>
       <c r="L16" s="63">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="M16" s="134">
+      <c r="M16" s="128">
         <f t="shared" si="1"/>
         <v>45820</v>
       </c>
-      <c r="N16" s="134"/>
+      <c r="N16" s="128"/>
       <c r="O16" s="64" t="str">
         <f t="shared" si="2"/>
         <v>qui</v>
       </c>
       <c r="P16" s="65"/>
-      <c r="Q16" s="130" t="s">
+      <c r="Q16" s="124" t="s">
         <v>95</v>
       </c>
-      <c r="R16" s="131"/>
+      <c r="R16" s="125"/>
     </row>
     <row r="17" spans="1:18" s="66" customFormat="1" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="57" t="s">
@@ -5946,23 +5714,23 @@
         <v>10</v>
       </c>
       <c r="E17" s="61"/>
-      <c r="F17" s="132"/>
-      <c r="G17" s="133"/>
+      <c r="F17" s="126"/>
+      <c r="G17" s="127"/>
       <c r="H17" s="62"/>
-      <c r="I17" s="132">
+      <c r="I17" s="126">
         <v>45818</v>
       </c>
-      <c r="J17" s="133"/>
+      <c r="J17" s="127"/>
       <c r="K17" s="62"/>
       <c r="L17" s="63">
         <f t="shared" si="0"/>
         <v>45818</v>
       </c>
-      <c r="M17" s="134">
+      <c r="M17" s="128">
         <f t="shared" si="1"/>
         <v>45828</v>
       </c>
-      <c r="N17" s="134"/>
+      <c r="N17" s="128"/>
       <c r="O17" s="64" t="str">
         <f t="shared" si="2"/>
         <v>sex</v>
@@ -5970,166 +5738,166 @@
       <c r="P17" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="Q17" s="130"/>
-      <c r="R17" s="131"/>
+      <c r="Q17" s="124"/>
+      <c r="R17" s="125"/>
     </row>
     <row r="18" spans="1:18" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="125" t="s">
+      <c r="B18" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="126"/>
+      <c r="C18" s="130"/>
       <c r="D18" s="41">
         <v>10</v>
       </c>
       <c r="E18" s="42"/>
-      <c r="F18" s="127">
+      <c r="F18" s="131">
         <v>45799</v>
       </c>
-      <c r="G18" s="128"/>
+      <c r="G18" s="132"/>
       <c r="H18" s="43"/>
-      <c r="I18" s="127">
+      <c r="I18" s="131">
         <v>45812</v>
       </c>
-      <c r="J18" s="128"/>
+      <c r="J18" s="132"/>
       <c r="K18" s="43"/>
       <c r="L18" s="44">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="M18" s="129">
+      <c r="M18" s="133">
         <f t="shared" si="1"/>
         <v>45821</v>
       </c>
-      <c r="N18" s="129"/>
+      <c r="N18" s="133"/>
       <c r="O18" s="45" t="str">
         <f t="shared" si="2"/>
         <v>sex</v>
       </c>
       <c r="P18" s="46"/>
-      <c r="Q18" s="130"/>
-      <c r="R18" s="131"/>
+      <c r="Q18" s="124"/>
+      <c r="R18" s="125"/>
     </row>
     <row r="19" spans="1:18" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="125" t="s">
+      <c r="B19" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="126"/>
+      <c r="C19" s="130"/>
       <c r="D19" s="41">
         <v>4</v>
       </c>
       <c r="E19" s="42"/>
-      <c r="F19" s="135">
+      <c r="F19" s="134">
         <v>45813</v>
       </c>
-      <c r="G19" s="136"/>
+      <c r="G19" s="135"/>
       <c r="H19" s="47"/>
-      <c r="I19" s="135">
+      <c r="I19" s="134">
         <v>45817</v>
       </c>
-      <c r="J19" s="136"/>
+      <c r="J19" s="135"/>
       <c r="K19" s="43"/>
       <c r="L19" s="44">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="M19" s="129">
+      <c r="M19" s="133">
         <f t="shared" si="1"/>
         <v>45821</v>
       </c>
-      <c r="N19" s="129"/>
+      <c r="N19" s="133"/>
       <c r="O19" s="45" t="str">
         <f t="shared" si="2"/>
         <v>sex</v>
       </c>
       <c r="P19" s="46"/>
-      <c r="Q19" s="130"/>
-      <c r="R19" s="131"/>
+      <c r="Q19" s="124"/>
+      <c r="R19" s="125"/>
     </row>
     <row r="20" spans="1:18" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="125" t="s">
+      <c r="B20" s="129" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="126"/>
+      <c r="C20" s="130"/>
       <c r="D20" s="41">
         <v>5</v>
       </c>
       <c r="E20" s="42"/>
-      <c r="F20" s="127">
+      <c r="F20" s="131">
         <v>45812</v>
       </c>
-      <c r="G20" s="128"/>
+      <c r="G20" s="132"/>
       <c r="H20" s="43"/>
-      <c r="I20" s="127">
+      <c r="I20" s="131">
         <v>45817</v>
       </c>
-      <c r="J20" s="128"/>
+      <c r="J20" s="132"/>
       <c r="K20" s="43"/>
       <c r="L20" s="44">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="M20" s="129">
+      <c r="M20" s="133">
         <f t="shared" si="1"/>
         <v>45821</v>
       </c>
-      <c r="N20" s="129"/>
+      <c r="N20" s="133"/>
       <c r="O20" s="45" t="str">
         <f t="shared" si="2"/>
         <v>sex</v>
       </c>
       <c r="P20" s="46"/>
-      <c r="Q20" s="130"/>
-      <c r="R20" s="131"/>
+      <c r="Q20" s="124"/>
+      <c r="R20" s="125"/>
     </row>
     <row r="21" spans="1:18" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="B21" s="125" t="s">
+      <c r="B21" s="129" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="126"/>
+      <c r="C21" s="130"/>
       <c r="D21" s="41">
         <v>10</v>
       </c>
       <c r="E21" s="42"/>
-      <c r="F21" s="127">
+      <c r="F21" s="131">
         <v>45807</v>
       </c>
-      <c r="G21" s="128"/>
+      <c r="G21" s="132"/>
       <c r="H21" s="43">
         <v>0</v>
       </c>
-      <c r="I21" s="127">
+      <c r="I21" s="131">
         <v>45819</v>
       </c>
-      <c r="J21" s="128"/>
+      <c r="J21" s="132"/>
       <c r="K21" s="43"/>
       <c r="L21" s="44">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="M21" s="129">
+      <c r="M21" s="133">
         <f t="shared" si="1"/>
         <v>45828</v>
       </c>
-      <c r="N21" s="129"/>
+      <c r="N21" s="133"/>
       <c r="O21" s="45" t="str">
         <f t="shared" si="2"/>
         <v>sex</v>
       </c>
       <c r="P21" s="46"/>
-      <c r="Q21" s="130"/>
-      <c r="R21" s="131"/>
+      <c r="Q21" s="124"/>
+      <c r="R21" s="125"/>
     </row>
     <row r="22" spans="1:18" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="16"/>
@@ -6142,35 +5910,35 @@
       <c r="O22" s="2"/>
     </row>
     <row r="23" spans="1:18" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="100" t="s">
+      <c r="A23" s="109" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="101"/>
-      <c r="C23" s="102"/>
+      <c r="B23" s="110"/>
+      <c r="C23" s="111"/>
       <c r="D23" s="20" t="s">
         <v>15</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="F23" s="95" t="s">
+      <c r="F23" s="112" t="s">
         <v>18</v>
       </c>
-      <c r="G23" s="96"/>
-      <c r="H23" s="97"/>
-      <c r="I23" s="95" t="s">
+      <c r="G23" s="113"/>
+      <c r="H23" s="114"/>
+      <c r="I23" s="112" t="s">
         <v>17</v>
       </c>
-      <c r="J23" s="96"/>
-      <c r="K23" s="97"/>
+      <c r="J23" s="113"/>
+      <c r="K23" s="114"/>
       <c r="L23" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="M23" s="109" t="s">
+      <c r="M23" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="N23" s="110"/>
-      <c r="O23" s="111"/>
+      <c r="N23" s="116"/>
+      <c r="O23" s="117"/>
       <c r="P23" s="15" t="s">
         <v>11</v>
       </c>
@@ -6179,10 +5947,10 @@
       <c r="A24" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="122" t="s">
+      <c r="B24" s="100" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="123"/>
+      <c r="C24" s="101"/>
       <c r="D24" s="18">
         <v>14</v>
       </c>
@@ -7134,10 +6902,10 @@
       <c r="A48" s="17">
         <v>109</v>
       </c>
-      <c r="B48" s="114" t="s">
+      <c r="B48" s="102" t="s">
         <v>42</v>
       </c>
-      <c r="C48" s="115"/>
+      <c r="C48" s="103"/>
       <c r="D48" s="18">
         <v>10</v>
       </c>
@@ -7173,10 +6941,10 @@
       <c r="A49" s="17">
         <v>110</v>
       </c>
-      <c r="B49" s="114" t="s">
+      <c r="B49" s="102" t="s">
         <v>43</v>
       </c>
-      <c r="C49" s="115"/>
+      <c r="C49" s="103"/>
       <c r="D49" s="18">
         <v>14</v>
       </c>
@@ -7212,10 +6980,10 @@
       <c r="A50" s="17">
         <v>1361</v>
       </c>
-      <c r="B50" s="114" t="s">
+      <c r="B50" s="102" t="s">
         <v>50</v>
       </c>
-      <c r="C50" s="115"/>
+      <c r="C50" s="103"/>
       <c r="D50" s="18">
         <v>25</v>
       </c>
@@ -7261,39 +7029,39 @@
       <c r="O51" s="8"/>
     </row>
     <row r="52" spans="1:18" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="109" t="str">
+      <c r="A52" s="115" t="str">
         <f>"Segunda(dia "&amp;TEXT($N$1+5,"DD")&amp;")"</f>
         <v>Segunda(dia 16)</v>
       </c>
-      <c r="B52" s="110"/>
-      <c r="C52" s="109" t="str">
+      <c r="B52" s="116"/>
+      <c r="C52" s="115" t="str">
         <f>"Terça(dia "&amp;TEXT($N$1+6,"DD")&amp;")"</f>
         <v>Terça(dia 17)</v>
       </c>
-      <c r="D52" s="110"/>
-      <c r="E52" s="110"/>
-      <c r="F52" s="111"/>
-      <c r="G52" s="110" t="str">
+      <c r="D52" s="116"/>
+      <c r="E52" s="116"/>
+      <c r="F52" s="117"/>
+      <c r="G52" s="116" t="str">
         <f>"Quarta(dia "&amp;TEXT($N$1+7,"DD")&amp;")"</f>
         <v>Quarta(dia 18)</v>
       </c>
-      <c r="H52" s="110"/>
-      <c r="I52" s="110"/>
-      <c r="J52" s="110"/>
-      <c r="K52" s="111"/>
-      <c r="L52" s="109" t="str">
+      <c r="H52" s="116"/>
+      <c r="I52" s="116"/>
+      <c r="J52" s="116"/>
+      <c r="K52" s="117"/>
+      <c r="L52" s="115" t="str">
         <f>"Quinta(dia "&amp;TEXT($N$1+8,"DD")&amp;")"</f>
         <v>Quinta(dia 19)</v>
       </c>
-      <c r="M52" s="110"/>
-      <c r="N52" s="110"/>
-      <c r="O52" s="110"/>
-      <c r="P52" s="111"/>
-      <c r="Q52" s="109" t="str">
+      <c r="M52" s="116"/>
+      <c r="N52" s="116"/>
+      <c r="O52" s="116"/>
+      <c r="P52" s="117"/>
+      <c r="Q52" s="115" t="str">
         <f>"Sexta(dia "&amp;TEXT($N$1+9,"DD")&amp;")"</f>
         <v>Sexta(dia 20)</v>
       </c>
-      <c r="R52" s="111"/>
+      <c r="R52" s="117"/>
     </row>
     <row r="53" spans="1:18" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="33" t="s">
@@ -7303,27 +7071,27 @@
         <v>59</v>
       </c>
       <c r="C53" s="35"/>
-      <c r="D53" s="124" t="s">
+      <c r="D53" s="136" t="s">
         <v>84</v>
       </c>
-      <c r="E53" s="124"/>
-      <c r="F53" s="124"/>
+      <c r="E53" s="136"/>
+      <c r="F53" s="136"/>
       <c r="G53" s="33" t="s">
         <v>96</v>
       </c>
-      <c r="H53" s="119" t="s">
+      <c r="H53" s="104" t="s">
         <v>92</v>
       </c>
-      <c r="I53" s="119"/>
-      <c r="J53" s="119"/>
-      <c r="K53" s="119"/>
+      <c r="I53" s="104"/>
+      <c r="J53" s="104"/>
+      <c r="K53" s="104"/>
       <c r="L53" s="36"/>
-      <c r="M53" s="124" t="s">
+      <c r="M53" s="136" t="s">
         <v>90</v>
       </c>
-      <c r="N53" s="124"/>
-      <c r="O53" s="124"/>
-      <c r="P53" s="124"/>
+      <c r="N53" s="136"/>
+      <c r="O53" s="136"/>
+      <c r="P53" s="136"/>
       <c r="Q53" s="33" t="s">
         <v>96</v>
       </c>
@@ -7339,25 +7107,25 @@
         <v>82</v>
       </c>
       <c r="C54" s="35"/>
-      <c r="D54" s="124" t="s">
+      <c r="D54" s="136" t="s">
         <v>85</v>
       </c>
-      <c r="E54" s="124"/>
-      <c r="F54" s="124"/>
+      <c r="E54" s="136"/>
+      <c r="F54" s="136"/>
       <c r="G54" s="36"/>
-      <c r="H54" s="124" t="s">
+      <c r="H54" s="136" t="s">
         <v>88</v>
       </c>
-      <c r="I54" s="124"/>
-      <c r="J54" s="124"/>
-      <c r="K54" s="124"/>
+      <c r="I54" s="136"/>
+      <c r="J54" s="136"/>
+      <c r="K54" s="136"/>
       <c r="L54" s="36"/>
-      <c r="M54" s="124" t="s">
+      <c r="M54" s="136" t="s">
         <v>89</v>
       </c>
-      <c r="N54" s="124"/>
-      <c r="O54" s="124"/>
-      <c r="P54" s="124"/>
+      <c r="N54" s="136"/>
+      <c r="O54" s="136"/>
+      <c r="P54" s="136"/>
       <c r="Q54" s="36"/>
       <c r="R54" s="2" t="str">
         <f>IFERROR(VLOOKUP(Q54,$A:$B,2,FALSE),"")</f>
@@ -7372,23 +7140,23 @@
         <v>83</v>
       </c>
       <c r="C55" s="35"/>
-      <c r="D55" s="124" t="s">
+      <c r="D55" s="136" t="s">
         <v>86</v>
       </c>
-      <c r="E55" s="124"/>
-      <c r="F55" s="124"/>
+      <c r="E55" s="136"/>
+      <c r="F55" s="136"/>
       <c r="G55" s="36"/>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
       <c r="L55" s="36"/>
-      <c r="M55" s="124" t="s">
+      <c r="M55" s="136" t="s">
         <v>93</v>
       </c>
-      <c r="N55" s="124"/>
-      <c r="O55" s="124"/>
-      <c r="P55" s="124"/>
+      <c r="N55" s="136"/>
+      <c r="O55" s="136"/>
+      <c r="P55" s="136"/>
       <c r="Q55" s="36"/>
       <c r="R55" s="2" t="str">
         <f>IFERROR(VLOOKUP(Q55,$A:$B,2,FALSE),"")</f>
@@ -7403,27 +7171,27 @@
         <v>90</v>
       </c>
       <c r="C56" s="36"/>
-      <c r="D56" s="124" t="s">
+      <c r="D56" s="136" t="s">
         <v>87</v>
       </c>
-      <c r="E56" s="124"/>
-      <c r="F56" s="124"/>
+      <c r="E56" s="136"/>
+      <c r="F56" s="136"/>
       <c r="G56" s="36"/>
-      <c r="H56" s="107" t="str">
+      <c r="H56" s="105" t="str">
         <f t="shared" ref="H56:H62" si="10">IFERROR(VLOOKUP(G56,$A:$B,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="I56" s="107"/>
-      <c r="J56" s="107"/>
-      <c r="K56" s="107"/>
+      <c r="I56" s="105"/>
+      <c r="J56" s="105"/>
+      <c r="K56" s="105"/>
       <c r="L56" s="36"/>
-      <c r="M56" s="119" t="str">
+      <c r="M56" s="104" t="str">
         <f t="shared" ref="M56:M70" si="11">IFERROR(VLOOKUP(L56,$A:$B,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="N56" s="119"/>
-      <c r="O56" s="119"/>
-      <c r="P56" s="119"/>
+      <c r="N56" s="104"/>
+      <c r="O56" s="104"/>
+      <c r="P56" s="104"/>
       <c r="Q56" s="36"/>
       <c r="R56" s="2" t="str">
         <f>IFERROR(VLOOKUP(Q56,$A:$B,2,FALSE),"")</f>
@@ -7438,27 +7206,27 @@
         <v>92</v>
       </c>
       <c r="C57" s="36"/>
-      <c r="D57" s="124" t="s">
+      <c r="D57" s="136" t="s">
         <v>94</v>
       </c>
-      <c r="E57" s="124"/>
-      <c r="F57" s="124"/>
+      <c r="E57" s="136"/>
+      <c r="F57" s="136"/>
       <c r="G57" s="36"/>
-      <c r="H57" s="119" t="str">
+      <c r="H57" s="104" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="I57" s="119"/>
-      <c r="J57" s="119"/>
-      <c r="K57" s="119"/>
+      <c r="I57" s="104"/>
+      <c r="J57" s="104"/>
+      <c r="K57" s="104"/>
       <c r="L57" s="36"/>
-      <c r="M57" s="119" t="str">
+      <c r="M57" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N57" s="119"/>
-      <c r="O57" s="119"/>
-      <c r="P57" s="119"/>
+      <c r="N57" s="104"/>
+      <c r="O57" s="104"/>
+      <c r="P57" s="104"/>
       <c r="Q57" s="36"/>
       <c r="R57" s="2" t="str">
         <f>IFERROR(VLOOKUP(Q57,$A:$B,2,FALSE),"")</f>
@@ -7472,28 +7240,28 @@
         <v/>
       </c>
       <c r="C58" s="36"/>
-      <c r="D58" s="107" t="str">
+      <c r="D58" s="105" t="str">
         <f t="shared" ref="D58:D63" si="13">IFERROR(VLOOKUP(C58,$A:$B,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="E58" s="107"/>
-      <c r="F58" s="107"/>
+      <c r="E58" s="105"/>
+      <c r="F58" s="105"/>
       <c r="G58" s="36"/>
-      <c r="H58" s="119" t="str">
+      <c r="H58" s="104" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="I58" s="119"/>
-      <c r="J58" s="119"/>
-      <c r="K58" s="119"/>
+      <c r="I58" s="104"/>
+      <c r="J58" s="104"/>
+      <c r="K58" s="104"/>
       <c r="L58" s="36"/>
-      <c r="M58" s="119" t="str">
+      <c r="M58" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N58" s="119"/>
-      <c r="O58" s="119"/>
-      <c r="P58" s="119"/>
+      <c r="N58" s="104"/>
+      <c r="O58" s="104"/>
+      <c r="P58" s="104"/>
       <c r="Q58" s="36"/>
       <c r="R58" s="2" t="str">
         <f t="shared" ref="R58:R70" si="14">IFERROR(VLOOKUP(Q58,$A:$B,2,FALSE),"")</f>
@@ -7507,28 +7275,28 @@
         <v/>
       </c>
       <c r="C59" s="36"/>
-      <c r="D59" s="107" t="str">
+      <c r="D59" s="105" t="str">
         <f t="shared" si="13"/>
         <v/>
       </c>
-      <c r="E59" s="107"/>
-      <c r="F59" s="107"/>
+      <c r="E59" s="105"/>
+      <c r="F59" s="105"/>
       <c r="G59" s="36"/>
-      <c r="H59" s="119" t="str">
+      <c r="H59" s="104" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="I59" s="119"/>
-      <c r="J59" s="119"/>
-      <c r="K59" s="119"/>
+      <c r="I59" s="104"/>
+      <c r="J59" s="104"/>
+      <c r="K59" s="104"/>
       <c r="L59" s="36"/>
-      <c r="M59" s="119" t="str">
+      <c r="M59" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N59" s="119"/>
-      <c r="O59" s="119"/>
-      <c r="P59" s="119"/>
+      <c r="N59" s="104"/>
+      <c r="O59" s="104"/>
+      <c r="P59" s="104"/>
       <c r="Q59" s="36"/>
       <c r="R59" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7542,28 +7310,28 @@
         <v/>
       </c>
       <c r="C60" s="36"/>
-      <c r="D60" s="107" t="str">
+      <c r="D60" s="105" t="str">
         <f t="shared" si="13"/>
         <v/>
       </c>
-      <c r="E60" s="107"/>
-      <c r="F60" s="107"/>
+      <c r="E60" s="105"/>
+      <c r="F60" s="105"/>
       <c r="G60" s="36"/>
-      <c r="H60" s="119" t="str">
+      <c r="H60" s="104" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="I60" s="119"/>
-      <c r="J60" s="119"/>
-      <c r="K60" s="119"/>
+      <c r="I60" s="104"/>
+      <c r="J60" s="104"/>
+      <c r="K60" s="104"/>
       <c r="L60" s="36"/>
-      <c r="M60" s="119" t="str">
+      <c r="M60" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N60" s="119"/>
-      <c r="O60" s="119"/>
-      <c r="P60" s="119"/>
+      <c r="N60" s="104"/>
+      <c r="O60" s="104"/>
+      <c r="P60" s="104"/>
       <c r="Q60" s="36"/>
       <c r="R60" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7577,28 +7345,28 @@
         <v/>
       </c>
       <c r="C61" s="36"/>
-      <c r="D61" s="107" t="str">
+      <c r="D61" s="105" t="str">
         <f t="shared" si="13"/>
         <v/>
       </c>
-      <c r="E61" s="107"/>
-      <c r="F61" s="107"/>
+      <c r="E61" s="105"/>
+      <c r="F61" s="105"/>
       <c r="G61" s="36"/>
-      <c r="H61" s="119" t="str">
+      <c r="H61" s="104" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="I61" s="119"/>
-      <c r="J61" s="119"/>
-      <c r="K61" s="119"/>
+      <c r="I61" s="104"/>
+      <c r="J61" s="104"/>
+      <c r="K61" s="104"/>
       <c r="L61" s="36"/>
-      <c r="M61" s="119" t="str">
+      <c r="M61" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N61" s="119"/>
-      <c r="O61" s="119"/>
-      <c r="P61" s="119"/>
+      <c r="N61" s="104"/>
+      <c r="O61" s="104"/>
+      <c r="P61" s="104"/>
       <c r="Q61" s="36"/>
       <c r="R61" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7612,28 +7380,28 @@
         <v/>
       </c>
       <c r="C62" s="36"/>
-      <c r="D62" s="107" t="str">
+      <c r="D62" s="105" t="str">
         <f t="shared" si="13"/>
         <v/>
       </c>
-      <c r="E62" s="107"/>
-      <c r="F62" s="107"/>
+      <c r="E62" s="105"/>
+      <c r="F62" s="105"/>
       <c r="G62" s="36"/>
-      <c r="H62" s="119" t="str">
+      <c r="H62" s="104" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="I62" s="119"/>
-      <c r="J62" s="119"/>
-      <c r="K62" s="119"/>
+      <c r="I62" s="104"/>
+      <c r="J62" s="104"/>
+      <c r="K62" s="104"/>
       <c r="L62" s="36"/>
-      <c r="M62" s="119" t="str">
+      <c r="M62" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N62" s="119"/>
-      <c r="O62" s="119"/>
-      <c r="P62" s="119"/>
+      <c r="N62" s="104"/>
+      <c r="O62" s="104"/>
+      <c r="P62" s="104"/>
       <c r="Q62" s="36"/>
       <c r="R62" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7647,28 +7415,28 @@
         <v/>
       </c>
       <c r="C63" s="36"/>
-      <c r="D63" s="107" t="str">
+      <c r="D63" s="105" t="str">
         <f t="shared" si="13"/>
         <v/>
       </c>
-      <c r="E63" s="107"/>
-      <c r="F63" s="107"/>
+      <c r="E63" s="105"/>
+      <c r="F63" s="105"/>
       <c r="G63" s="36"/>
-      <c r="H63" s="119" t="str">
+      <c r="H63" s="104" t="str">
         <f t="shared" ref="H63:H70" si="15">IFERROR(VLOOKUP(G63,$A:$B,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="I63" s="119"/>
-      <c r="J63" s="119"/>
-      <c r="K63" s="119"/>
+      <c r="I63" s="104"/>
+      <c r="J63" s="104"/>
+      <c r="K63" s="104"/>
       <c r="L63" s="36"/>
-      <c r="M63" s="119" t="str">
+      <c r="M63" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N63" s="119"/>
-      <c r="O63" s="119"/>
-      <c r="P63" s="119"/>
+      <c r="N63" s="104"/>
+      <c r="O63" s="104"/>
+      <c r="P63" s="104"/>
       <c r="Q63" s="36"/>
       <c r="R63" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7682,28 +7450,28 @@
         <v/>
       </c>
       <c r="C64" s="36"/>
-      <c r="D64" s="119" t="str">
+      <c r="D64" s="104" t="str">
         <f t="shared" ref="D64:D70" si="16">IFERROR(VLOOKUP(C64,$A:$B,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="E64" s="119"/>
-      <c r="F64" s="119"/>
+      <c r="E64" s="104"/>
+      <c r="F64" s="104"/>
       <c r="G64" s="36"/>
-      <c r="H64" s="119" t="str">
+      <c r="H64" s="104" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="I64" s="119"/>
-      <c r="J64" s="119"/>
-      <c r="K64" s="119"/>
+      <c r="I64" s="104"/>
+      <c r="J64" s="104"/>
+      <c r="K64" s="104"/>
       <c r="L64" s="36"/>
-      <c r="M64" s="119" t="str">
+      <c r="M64" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N64" s="119"/>
-      <c r="O64" s="119"/>
-      <c r="P64" s="119"/>
+      <c r="N64" s="104"/>
+      <c r="O64" s="104"/>
+      <c r="P64" s="104"/>
       <c r="Q64" s="37"/>
       <c r="R64" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7717,28 +7485,28 @@
         <v/>
       </c>
       <c r="C65" s="37"/>
-      <c r="D65" s="119" t="str">
+      <c r="D65" s="104" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="E65" s="119"/>
-      <c r="F65" s="119"/>
+      <c r="E65" s="104"/>
+      <c r="F65" s="104"/>
       <c r="G65" s="36"/>
-      <c r="H65" s="119" t="str">
+      <c r="H65" s="104" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="I65" s="119"/>
-      <c r="J65" s="119"/>
-      <c r="K65" s="119"/>
+      <c r="I65" s="104"/>
+      <c r="J65" s="104"/>
+      <c r="K65" s="104"/>
       <c r="L65" s="38"/>
-      <c r="M65" s="119" t="str">
+      <c r="M65" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N65" s="119"/>
-      <c r="O65" s="119"/>
-      <c r="P65" s="119"/>
+      <c r="N65" s="104"/>
+      <c r="O65" s="104"/>
+      <c r="P65" s="104"/>
       <c r="Q65" s="37"/>
       <c r="R65" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7752,28 +7520,28 @@
         <v/>
       </c>
       <c r="C66" s="37"/>
-      <c r="D66" s="119" t="str">
+      <c r="D66" s="104" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="E66" s="119"/>
-      <c r="F66" s="119"/>
+      <c r="E66" s="104"/>
+      <c r="F66" s="104"/>
       <c r="G66" s="36"/>
-      <c r="H66" s="119" t="str">
+      <c r="H66" s="104" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="I66" s="119"/>
-      <c r="J66" s="119"/>
-      <c r="K66" s="119"/>
+      <c r="I66" s="104"/>
+      <c r="J66" s="104"/>
+      <c r="K66" s="104"/>
       <c r="L66" s="38"/>
-      <c r="M66" s="119" t="str">
+      <c r="M66" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N66" s="119"/>
-      <c r="O66" s="119"/>
-      <c r="P66" s="119"/>
+      <c r="N66" s="104"/>
+      <c r="O66" s="104"/>
+      <c r="P66" s="104"/>
       <c r="Q66" s="37"/>
       <c r="R66" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7787,28 +7555,28 @@
         <v/>
       </c>
       <c r="C67" s="37"/>
-      <c r="D67" s="119" t="str">
+      <c r="D67" s="104" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="E67" s="119"/>
-      <c r="F67" s="119"/>
+      <c r="E67" s="104"/>
+      <c r="F67" s="104"/>
       <c r="G67" s="36"/>
-      <c r="H67" s="119" t="str">
+      <c r="H67" s="104" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="I67" s="119"/>
-      <c r="J67" s="119"/>
-      <c r="K67" s="119"/>
+      <c r="I67" s="104"/>
+      <c r="J67" s="104"/>
+      <c r="K67" s="104"/>
       <c r="L67" s="38"/>
-      <c r="M67" s="119" t="str">
+      <c r="M67" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N67" s="119"/>
-      <c r="O67" s="119"/>
-      <c r="P67" s="119"/>
+      <c r="N67" s="104"/>
+      <c r="O67" s="104"/>
+      <c r="P67" s="104"/>
       <c r="Q67" s="37"/>
       <c r="R67" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7818,28 +7586,28 @@
     <row r="68" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="37"/>
       <c r="C68" s="37"/>
-      <c r="D68" s="119" t="str">
+      <c r="D68" s="104" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="E68" s="119"/>
-      <c r="F68" s="119"/>
+      <c r="E68" s="104"/>
+      <c r="F68" s="104"/>
       <c r="G68" s="36"/>
-      <c r="H68" s="119" t="str">
+      <c r="H68" s="104" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="I68" s="119"/>
-      <c r="J68" s="119"/>
-      <c r="K68" s="119"/>
+      <c r="I68" s="104"/>
+      <c r="J68" s="104"/>
+      <c r="K68" s="104"/>
       <c r="L68" s="38"/>
-      <c r="M68" s="119" t="str">
+      <c r="M68" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N68" s="119"/>
-      <c r="O68" s="119"/>
-      <c r="P68" s="119"/>
+      <c r="N68" s="104"/>
+      <c r="O68" s="104"/>
+      <c r="P68" s="104"/>
       <c r="Q68" s="37"/>
       <c r="R68" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7853,28 +7621,28 @@
         <v/>
       </c>
       <c r="C69" s="37"/>
-      <c r="D69" s="119" t="str">
+      <c r="D69" s="104" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="E69" s="119"/>
-      <c r="F69" s="119"/>
+      <c r="E69" s="104"/>
+      <c r="F69" s="104"/>
       <c r="G69" s="36"/>
-      <c r="H69" s="119" t="str">
+      <c r="H69" s="104" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="I69" s="119"/>
-      <c r="J69" s="119"/>
-      <c r="K69" s="119"/>
+      <c r="I69" s="104"/>
+      <c r="J69" s="104"/>
+      <c r="K69" s="104"/>
       <c r="L69" s="38"/>
-      <c r="M69" s="119" t="str">
+      <c r="M69" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N69" s="119"/>
-      <c r="O69" s="119"/>
-      <c r="P69" s="119"/>
+      <c r="N69" s="104"/>
+      <c r="O69" s="104"/>
+      <c r="P69" s="104"/>
       <c r="Q69" s="37"/>
       <c r="R69" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7888,28 +7656,28 @@
         <v/>
       </c>
       <c r="C70" s="37"/>
-      <c r="D70" s="119" t="str">
+      <c r="D70" s="104" t="str">
         <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="E70" s="119"/>
-      <c r="F70" s="119"/>
+      <c r="E70" s="104"/>
+      <c r="F70" s="104"/>
       <c r="G70" s="36"/>
-      <c r="H70" s="119" t="str">
+      <c r="H70" s="104" t="str">
         <f t="shared" si="15"/>
         <v/>
       </c>
-      <c r="I70" s="119"/>
-      <c r="J70" s="119"/>
-      <c r="K70" s="119"/>
+      <c r="I70" s="104"/>
+      <c r="J70" s="104"/>
+      <c r="K70" s="104"/>
       <c r="L70" s="38"/>
-      <c r="M70" s="119" t="str">
+      <c r="M70" s="104" t="str">
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="N70" s="119"/>
-      <c r="O70" s="119"/>
-      <c r="P70" s="119"/>
+      <c r="N70" s="104"/>
+      <c r="O70" s="104"/>
+      <c r="P70" s="104"/>
       <c r="Q70" s="37"/>
       <c r="R70" s="2" t="str">
         <f t="shared" si="14"/>
@@ -7968,45 +7736,161 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" deleteColumns="0" deleteRows="0" sort="0"/>
   <mergeCells count="216">
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="M2:O2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="I3:J3"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="D69:F69"/>
+    <mergeCell ref="H69:K69"/>
+    <mergeCell ref="M69:P69"/>
+    <mergeCell ref="D70:F70"/>
+    <mergeCell ref="H70:K70"/>
+    <mergeCell ref="M70:P70"/>
+    <mergeCell ref="D67:F67"/>
+    <mergeCell ref="H67:K67"/>
+    <mergeCell ref="M67:P67"/>
+    <mergeCell ref="D68:F68"/>
+    <mergeCell ref="H68:K68"/>
+    <mergeCell ref="M68:P68"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="H65:K65"/>
+    <mergeCell ref="M65:P65"/>
+    <mergeCell ref="D66:F66"/>
+    <mergeCell ref="H66:K66"/>
+    <mergeCell ref="M66:P66"/>
+    <mergeCell ref="D63:F63"/>
+    <mergeCell ref="H63:K63"/>
+    <mergeCell ref="M63:P63"/>
+    <mergeCell ref="D64:F64"/>
+    <mergeCell ref="H64:K64"/>
+    <mergeCell ref="M64:P64"/>
+    <mergeCell ref="D61:F61"/>
+    <mergeCell ref="H61:K61"/>
+    <mergeCell ref="M61:P61"/>
+    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="H62:K62"/>
+    <mergeCell ref="M62:P62"/>
+    <mergeCell ref="D59:F59"/>
+    <mergeCell ref="H59:K59"/>
+    <mergeCell ref="M59:P59"/>
+    <mergeCell ref="D60:F60"/>
+    <mergeCell ref="H60:K60"/>
+    <mergeCell ref="M60:P60"/>
+    <mergeCell ref="D57:F57"/>
+    <mergeCell ref="H57:K57"/>
+    <mergeCell ref="M57:P57"/>
+    <mergeCell ref="D58:F58"/>
+    <mergeCell ref="H58:K58"/>
+    <mergeCell ref="M58:P58"/>
+    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="H54:K54"/>
+    <mergeCell ref="M54:P54"/>
+    <mergeCell ref="D55:F55"/>
+    <mergeCell ref="M55:P55"/>
+    <mergeCell ref="D56:F56"/>
+    <mergeCell ref="H56:K56"/>
+    <mergeCell ref="M56:P56"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="C52:F52"/>
+    <mergeCell ref="G52:K52"/>
+    <mergeCell ref="L52:P52"/>
+    <mergeCell ref="Q52:R52"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="H53:K53"/>
+    <mergeCell ref="M53:P53"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="M49:N49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="M50:N50"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="M47:N47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="M48:N48"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="M45:N45"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="M46:N46"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="M43:N43"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="M44:N44"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="M41:N41"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="M42:N42"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="M39:N39"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="M40:N40"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="M37:N37"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="M35:N35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="M36:N36"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="M27:N27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="M26:N26"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="M23:O23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="M21:N21"/>
     <mergeCell ref="Q16:R21"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="I17:J17"/>
@@ -8029,161 +7913,45 @@
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="I16:J16"/>
     <mergeCell ref="M16:N16"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="M23:O23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="M26:N26"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="M31:N31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="M29:N29"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="M30:N30"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="M35:N35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="M36:N36"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="M39:N39"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="M40:N40"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="M37:N37"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="M43:N43"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="M41:N41"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="M42:N42"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="M47:N47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="M48:N48"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="M45:N45"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="M46:N46"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="C52:F52"/>
-    <mergeCell ref="G52:K52"/>
-    <mergeCell ref="L52:P52"/>
-    <mergeCell ref="Q52:R52"/>
-    <mergeCell ref="D53:F53"/>
-    <mergeCell ref="H53:K53"/>
-    <mergeCell ref="M53:P53"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="M49:N49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="M50:N50"/>
-    <mergeCell ref="D57:F57"/>
-    <mergeCell ref="H57:K57"/>
-    <mergeCell ref="M57:P57"/>
-    <mergeCell ref="D58:F58"/>
-    <mergeCell ref="H58:K58"/>
-    <mergeCell ref="M58:P58"/>
-    <mergeCell ref="D54:F54"/>
-    <mergeCell ref="H54:K54"/>
-    <mergeCell ref="M54:P54"/>
-    <mergeCell ref="D55:F55"/>
-    <mergeCell ref="M55:P55"/>
-    <mergeCell ref="D56:F56"/>
-    <mergeCell ref="H56:K56"/>
-    <mergeCell ref="M56:P56"/>
-    <mergeCell ref="D61:F61"/>
-    <mergeCell ref="H61:K61"/>
-    <mergeCell ref="M61:P61"/>
-    <mergeCell ref="D62:F62"/>
-    <mergeCell ref="H62:K62"/>
-    <mergeCell ref="M62:P62"/>
-    <mergeCell ref="D59:F59"/>
-    <mergeCell ref="H59:K59"/>
-    <mergeCell ref="M59:P59"/>
-    <mergeCell ref="D60:F60"/>
-    <mergeCell ref="H60:K60"/>
-    <mergeCell ref="M60:P60"/>
-    <mergeCell ref="D65:F65"/>
-    <mergeCell ref="H65:K65"/>
-    <mergeCell ref="M65:P65"/>
-    <mergeCell ref="D66:F66"/>
-    <mergeCell ref="H66:K66"/>
-    <mergeCell ref="M66:P66"/>
-    <mergeCell ref="D63:F63"/>
-    <mergeCell ref="H63:K63"/>
-    <mergeCell ref="M63:P63"/>
-    <mergeCell ref="D64:F64"/>
-    <mergeCell ref="H64:K64"/>
-    <mergeCell ref="M64:P64"/>
-    <mergeCell ref="D69:F69"/>
-    <mergeCell ref="H69:K69"/>
-    <mergeCell ref="M69:P69"/>
-    <mergeCell ref="D70:F70"/>
-    <mergeCell ref="H70:K70"/>
-    <mergeCell ref="M70:P70"/>
-    <mergeCell ref="D67:F67"/>
-    <mergeCell ref="H67:K67"/>
-    <mergeCell ref="M67:P67"/>
-    <mergeCell ref="D68:F68"/>
-    <mergeCell ref="H68:K68"/>
-    <mergeCell ref="M68:P68"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="M2:O2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="M6:N6"/>
   </mergeCells>
   <conditionalFormatting sqref="M3:O21 M24:O50">
     <cfRule type="expression" dxfId="3" priority="2">

</xml_diff>